<commit_message>
MTP106 done; COP row summary file checker improved with delta seconds between COP file and summary for quicker checking
</commit_message>
<xml_diff>
--- a/observations/calibrations/solar_calibrations.xlsx
+++ b/observations/calibrations/solar_calibrations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iant\Documents\PROGRAMS\nomad_obs\observations\calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB7ADF0C-B060-4E32-8BD1-0E8BBD1A0E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77CC3814-7648-4D5A-A5A1-1AFE76ECCB67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -911,7 +911,7 @@
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1022,11 +1022,13 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="26" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1037,6 +1039,35 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1360,7 +1391,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE147"/>
+  <dimension ref="A1:AE150"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.5546875" bestFit="1" customWidth="1"/>
@@ -4690,36 +4721,42 @@
       <c r="A88">
         <v>4</v>
       </c>
-      <c r="B88" s="5">
+      <c r="B88" s="38">
         <v>119</v>
       </c>
       <c r="C88" s="44">
         <v>386</v>
       </c>
-      <c r="D88" s="58">
+      <c r="D88" s="108">
         <v>370</v>
       </c>
-      <c r="E88">
+      <c r="E88" s="26">
         <v>189</v>
       </c>
-      <c r="F88" s="2">
+      <c r="F88" s="15">
         <v>100</v>
       </c>
-      <c r="J88" s="4"/>
-      <c r="L88" s="5">
+      <c r="G88" s="16"/>
+      <c r="H88" s="16"/>
+      <c r="I88" s="16"/>
+      <c r="J88" s="17"/>
+      <c r="L88" s="38">
         <v>119</v>
       </c>
-      <c r="M88" s="42">
+      <c r="M88" s="44">
         <v>419</v>
       </c>
       <c r="N88" s="58">
         <v>403</v>
       </c>
-      <c r="O88">
+      <c r="O88" s="16">
         <v>236</v>
       </c>
-      <c r="P88" s="5"/>
-      <c r="T88" s="4"/>
+      <c r="P88" s="38"/>
+      <c r="Q88" s="16"/>
+      <c r="R88" s="16"/>
+      <c r="S88" s="16"/>
+      <c r="T88" s="17"/>
     </row>
     <row r="89" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A89">
@@ -4733,36 +4770,41 @@
         <f>C88+2</f>
         <v>388</v>
       </c>
-      <c r="D89" s="59">
+      <c r="D89" s="97">
         <v>371</v>
       </c>
-      <c r="E89">
+      <c r="E89" s="25">
         <v>190</v>
       </c>
-      <c r="F89" s="2">
+      <c r="F89" s="98">
         <v>9</v>
       </c>
-      <c r="G89" s="3">
+      <c r="G89" s="98">
         <v>80</v>
       </c>
+      <c r="H89" s="95"/>
+      <c r="I89" s="95"/>
       <c r="J89" s="4"/>
       <c r="L89" s="5">
         <f>L88+3</f>
         <v>122</v>
       </c>
       <c r="M89" s="42">
-        <f t="shared" ref="M89:M116" si="4">M88+2</f>
+        <f t="shared" ref="M89:M115" si="4">M88+2</f>
         <v>421</v>
       </c>
       <c r="N89" s="59">
         <v>404</v>
       </c>
-      <c r="O89">
+      <c r="O89" s="95">
         <v>237</v>
       </c>
       <c r="P89" s="2">
         <v>9</v>
       </c>
+      <c r="Q89" s="95"/>
+      <c r="R89" s="95"/>
+      <c r="S89" s="95"/>
       <c r="T89" s="4"/>
     </row>
     <row r="90" spans="1:20" x14ac:dyDescent="0.3">
@@ -4770,33 +4812,33 @@
         <v>4</v>
       </c>
       <c r="B90" s="29">
-        <f t="shared" ref="B90:B116" si="5">B89+3</f>
+        <f t="shared" ref="B90:B115" si="5">B89+3</f>
         <v>125</v>
       </c>
       <c r="C90" s="41">
-        <f t="shared" ref="C90:C116" si="6">C89+2</f>
+        <f t="shared" ref="C90:C115" si="6">C89+2</f>
         <v>390</v>
       </c>
-      <c r="D90" s="60">
+      <c r="D90" s="109">
         <v>372</v>
       </c>
-      <c r="E90" s="3">
+      <c r="E90" s="107">
         <v>191</v>
       </c>
-      <c r="F90" s="29">
+      <c r="F90" s="99">
         <v>7</v>
       </c>
-      <c r="G90" s="32">
+      <c r="G90" s="99">
         <v>57</v>
       </c>
-      <c r="H90" s="32">
+      <c r="H90" s="99">
         <v>80</v>
       </c>
-      <c r="I90" s="30"/>
+      <c r="I90" s="100"/>
       <c r="J90" s="31"/>
       <c r="K90" s="30"/>
       <c r="L90" s="29">
-        <f t="shared" ref="L90:L116" si="7">L89+3</f>
+        <f t="shared" ref="L90:L115" si="7">L89+3</f>
         <v>125</v>
       </c>
       <c r="M90" s="41">
@@ -4806,15 +4848,15 @@
       <c r="N90" s="60">
         <v>405</v>
       </c>
-      <c r="O90" s="3">
+      <c r="O90" s="98">
         <v>238</v>
       </c>
       <c r="P90" s="29">
         <v>7</v>
       </c>
-      <c r="Q90" s="30"/>
-      <c r="R90" s="30"/>
-      <c r="S90" s="30"/>
+      <c r="Q90" s="100"/>
+      <c r="R90" s="100"/>
+      <c r="S90" s="100"/>
       <c r="T90" s="31"/>
     </row>
     <row r="91" spans="1:20" x14ac:dyDescent="0.3">
@@ -4829,22 +4871,22 @@
         <f t="shared" si="6"/>
         <v>392</v>
       </c>
-      <c r="D91" s="75">
+      <c r="D91" s="110">
         <v>373</v>
       </c>
-      <c r="E91" s="73">
+      <c r="E91" s="74">
         <v>192</v>
       </c>
-      <c r="F91" s="81">
+      <c r="F91" s="102">
         <v>57</v>
       </c>
-      <c r="G91" s="79">
+      <c r="G91" s="102">
         <v>81</v>
       </c>
-      <c r="H91" s="79">
+      <c r="H91" s="102">
         <v>86</v>
       </c>
-      <c r="I91" s="73"/>
+      <c r="I91" s="101"/>
       <c r="J91" s="85"/>
       <c r="L91" s="35">
         <f t="shared" si="7"/>
@@ -4857,12 +4899,15 @@
       <c r="N91" s="75">
         <v>406</v>
       </c>
-      <c r="O91" s="73">
+      <c r="O91" s="101">
         <v>239</v>
       </c>
       <c r="P91" s="5">
         <v>60</v>
       </c>
+      <c r="Q91" s="95"/>
+      <c r="R91" s="95"/>
+      <c r="S91" s="95"/>
       <c r="T91" s="4"/>
     </row>
     <row r="92" spans="1:20" x14ac:dyDescent="0.3">
@@ -4877,15 +4922,18 @@
         <f t="shared" si="6"/>
         <v>394</v>
       </c>
-      <c r="D92" s="59">
+      <c r="D92" s="97">
         <v>374</v>
       </c>
-      <c r="E92">
+      <c r="E92" s="25">
         <v>193</v>
       </c>
-      <c r="F92" s="2">
+      <c r="F92" s="98">
         <v>81</v>
       </c>
+      <c r="G92" s="95"/>
+      <c r="H92" s="95"/>
+      <c r="I92" s="95"/>
       <c r="J92" s="4"/>
       <c r="L92" s="5">
         <f t="shared" si="7"/>
@@ -4898,10 +4946,13 @@
       <c r="N92" s="59">
         <v>407</v>
       </c>
-      <c r="O92">
+      <c r="O92" s="95">
         <v>240</v>
       </c>
       <c r="P92" s="5"/>
+      <c r="Q92" s="95"/>
+      <c r="R92" s="95"/>
+      <c r="S92" s="95"/>
       <c r="T92" s="4"/>
     </row>
     <row r="93" spans="1:20" x14ac:dyDescent="0.3">
@@ -4916,15 +4967,18 @@
         <f t="shared" si="6"/>
         <v>396</v>
       </c>
-      <c r="D93" s="59">
+      <c r="D93" s="97">
         <v>375</v>
       </c>
-      <c r="E93">
+      <c r="E93" s="25">
         <v>194</v>
       </c>
-      <c r="F93" s="2">
+      <c r="F93" s="98">
         <v>100</v>
       </c>
+      <c r="G93" s="95"/>
+      <c r="H93" s="95"/>
+      <c r="I93" s="95"/>
       <c r="J93" s="4"/>
       <c r="L93" s="5">
         <f t="shared" si="7"/>
@@ -4937,10 +4991,13 @@
       <c r="N93" s="59">
         <v>408</v>
       </c>
-      <c r="O93">
+      <c r="O93" s="95">
         <v>241</v>
       </c>
       <c r="P93" s="5"/>
+      <c r="Q93" s="95"/>
+      <c r="R93" s="95"/>
+      <c r="S93" s="95"/>
       <c r="T93" s="4"/>
     </row>
     <row r="94" spans="1:20" x14ac:dyDescent="0.3">
@@ -4955,18 +5012,20 @@
         <f t="shared" si="6"/>
         <v>398</v>
       </c>
-      <c r="D94" s="59">
+      <c r="D94" s="97">
         <v>376</v>
       </c>
-      <c r="E94">
+      <c r="E94" s="25">
         <v>195</v>
       </c>
-      <c r="F94" s="2">
+      <c r="F94" s="98">
         <v>9</v>
       </c>
-      <c r="G94" s="3">
+      <c r="G94" s="98">
         <v>82</v>
       </c>
+      <c r="H94" s="95"/>
+      <c r="I94" s="95"/>
       <c r="J94" s="4"/>
       <c r="L94" s="5">
         <f t="shared" si="7"/>
@@ -4979,12 +5038,15 @@
       <c r="N94" s="59">
         <v>409</v>
       </c>
-      <c r="O94">
+      <c r="O94" s="95">
         <v>242</v>
       </c>
       <c r="P94" s="2">
         <v>9</v>
       </c>
+      <c r="Q94" s="95"/>
+      <c r="R94" s="95"/>
+      <c r="S94" s="95"/>
       <c r="T94" s="4"/>
     </row>
     <row r="95" spans="1:20" x14ac:dyDescent="0.3">
@@ -4999,23 +5061,23 @@
         <f t="shared" si="6"/>
         <v>400</v>
       </c>
-      <c r="D95" s="78">
+      <c r="D95" s="111">
         <v>377</v>
       </c>
-      <c r="E95" s="79">
+      <c r="E95" s="77">
         <v>196</v>
       </c>
-      <c r="F95" s="80">
+      <c r="F95" s="103">
         <v>7</v>
       </c>
-      <c r="G95" s="82">
+      <c r="G95" s="103">
         <v>15</v>
       </c>
-      <c r="H95" s="82">
+      <c r="H95" s="103">
         <v>82</v>
       </c>
-      <c r="I95" s="87"/>
-      <c r="J95" s="88"/>
+      <c r="I95" s="104"/>
+      <c r="J95" s="86"/>
       <c r="K95" s="30"/>
       <c r="L95" s="80">
         <f t="shared" si="7"/>
@@ -5028,17 +5090,17 @@
       <c r="N95" s="78">
         <v>410</v>
       </c>
-      <c r="O95" s="79">
+      <c r="O95" s="102">
         <v>243</v>
       </c>
       <c r="P95" s="29">
         <v>7</v>
       </c>
-      <c r="Q95" s="32">
+      <c r="Q95" s="99">
         <v>15</v>
       </c>
-      <c r="R95" s="30"/>
-      <c r="S95" s="30"/>
+      <c r="R95" s="100"/>
+      <c r="S95" s="100"/>
       <c r="T95" s="31"/>
     </row>
     <row r="96" spans="1:20" x14ac:dyDescent="0.3">
@@ -5053,15 +5115,18 @@
         <f t="shared" si="6"/>
         <v>402</v>
       </c>
-      <c r="D96" s="59">
+      <c r="D96" s="97">
         <v>378</v>
       </c>
-      <c r="E96">
+      <c r="E96" s="25">
         <v>197</v>
       </c>
-      <c r="F96" s="2">
+      <c r="F96" s="98">
         <v>82</v>
       </c>
+      <c r="G96" s="95"/>
+      <c r="H96" s="95"/>
+      <c r="I96" s="95"/>
       <c r="J96" s="4"/>
       <c r="L96" s="5">
         <f t="shared" si="7"/>
@@ -5074,12 +5139,15 @@
       <c r="N96" s="59">
         <v>411</v>
       </c>
-      <c r="O96">
+      <c r="O96" s="95">
         <v>244</v>
       </c>
       <c r="P96" s="2">
         <v>39</v>
       </c>
+      <c r="Q96" s="95"/>
+      <c r="R96" s="95"/>
+      <c r="S96" s="95"/>
       <c r="T96" s="4"/>
     </row>
     <row r="97" spans="1:20" x14ac:dyDescent="0.3">
@@ -5094,23 +5162,23 @@
         <f t="shared" si="6"/>
         <v>404</v>
       </c>
-      <c r="D97" s="78">
+      <c r="D97" s="111">
         <v>379</v>
       </c>
-      <c r="E97" s="79">
+      <c r="E97" s="77">
         <v>198</v>
       </c>
-      <c r="F97" s="80">
+      <c r="F97" s="103">
         <v>8</v>
       </c>
-      <c r="G97" s="82">
+      <c r="G97" s="103">
         <v>21</v>
       </c>
-      <c r="H97" s="82">
+      <c r="H97" s="103">
         <v>82</v>
       </c>
-      <c r="I97" s="87"/>
-      <c r="J97" s="88"/>
+      <c r="I97" s="104"/>
+      <c r="J97" s="86"/>
       <c r="K97" s="30"/>
       <c r="L97" s="80">
         <f t="shared" si="7"/>
@@ -5123,15 +5191,15 @@
       <c r="N97" s="78">
         <v>412</v>
       </c>
-      <c r="O97" s="79">
+      <c r="O97" s="102">
         <v>245</v>
       </c>
       <c r="P97" s="29">
         <v>8</v>
       </c>
-      <c r="Q97" s="30"/>
-      <c r="R97" s="30"/>
-      <c r="S97" s="30"/>
+      <c r="Q97" s="100"/>
+      <c r="R97" s="100"/>
+      <c r="S97" s="100"/>
       <c r="T97" s="31"/>
     </row>
     <row r="98" spans="1:20" x14ac:dyDescent="0.3">
@@ -5146,20 +5214,20 @@
         <f t="shared" si="6"/>
         <v>406</v>
       </c>
-      <c r="D98" s="60">
+      <c r="D98" s="109">
         <v>380</v>
       </c>
-      <c r="E98" s="3">
+      <c r="E98" s="107">
         <v>199</v>
       </c>
-      <c r="F98" s="29">
+      <c r="F98" s="99">
         <v>23</v>
       </c>
-      <c r="G98" s="32">
+      <c r="G98" s="99">
         <v>86</v>
       </c>
-      <c r="H98" s="30"/>
-      <c r="I98" s="30"/>
+      <c r="H98" s="100"/>
+      <c r="I98" s="100"/>
       <c r="J98" s="31"/>
       <c r="L98" s="29">
         <f t="shared" si="7"/>
@@ -5172,15 +5240,15 @@
       <c r="N98" s="60">
         <v>413</v>
       </c>
-      <c r="O98" s="3">
+      <c r="O98" s="98">
         <v>246</v>
       </c>
       <c r="P98" s="28">
         <v>60</v>
       </c>
-      <c r="Q98" s="30"/>
-      <c r="R98" s="30"/>
-      <c r="S98" s="30"/>
+      <c r="Q98" s="100"/>
+      <c r="R98" s="100"/>
+      <c r="S98" s="100"/>
       <c r="T98" s="31"/>
     </row>
     <row r="99" spans="1:20" x14ac:dyDescent="0.3">
@@ -5195,15 +5263,18 @@
         <f t="shared" si="6"/>
         <v>408</v>
       </c>
-      <c r="D99" s="59">
+      <c r="D99" s="97">
         <v>381</v>
       </c>
-      <c r="E99">
+      <c r="E99" s="25">
         <v>200</v>
       </c>
-      <c r="F99" s="86">
+      <c r="F99" s="106">
         <v>100</v>
       </c>
+      <c r="G99" s="95"/>
+      <c r="H99" s="95"/>
+      <c r="I99" s="95"/>
       <c r="J99" s="4"/>
       <c r="L99" s="5">
         <f t="shared" si="7"/>
@@ -5216,12 +5287,15 @@
       <c r="N99" s="59">
         <v>414</v>
       </c>
-      <c r="O99">
+      <c r="O99" s="95">
         <v>247</v>
       </c>
       <c r="P99" s="35">
         <v>60</v>
       </c>
+      <c r="Q99" s="95"/>
+      <c r="R99" s="95"/>
+      <c r="S99" s="95"/>
       <c r="T99" s="4"/>
     </row>
     <row r="100" spans="1:20" x14ac:dyDescent="0.3">
@@ -5236,15 +5310,18 @@
         <f t="shared" si="6"/>
         <v>410</v>
       </c>
-      <c r="D100" s="59">
+      <c r="D100" s="97">
         <v>382</v>
       </c>
-      <c r="E100">
+      <c r="E100" s="25">
         <v>201</v>
       </c>
-      <c r="F100" s="2">
+      <c r="F100" s="98">
         <v>100</v>
       </c>
+      <c r="G100" s="95"/>
+      <c r="H100" s="95"/>
+      <c r="I100" s="95"/>
       <c r="J100" s="4"/>
       <c r="L100" s="5">
         <f t="shared" si="7"/>
@@ -5257,12 +5334,15 @@
       <c r="N100" s="59">
         <v>415</v>
       </c>
-      <c r="O100">
+      <c r="O100" s="95">
         <v>248</v>
       </c>
       <c r="P100" s="5">
         <v>60</v>
       </c>
+      <c r="Q100" s="95"/>
+      <c r="R100" s="95"/>
+      <c r="S100" s="95"/>
       <c r="T100" s="4"/>
     </row>
     <row r="101" spans="1:20" x14ac:dyDescent="0.3">
@@ -5277,15 +5357,18 @@
         <f t="shared" si="6"/>
         <v>412</v>
       </c>
-      <c r="D101" s="59">
+      <c r="D101" s="97">
         <v>383</v>
       </c>
-      <c r="E101">
+      <c r="E101" s="25">
         <v>202</v>
       </c>
-      <c r="F101" s="2">
+      <c r="F101" s="98">
         <v>9</v>
       </c>
+      <c r="G101" s="95"/>
+      <c r="H101" s="95"/>
+      <c r="I101" s="95"/>
       <c r="J101" s="4"/>
       <c r="L101" s="5">
         <f t="shared" si="7"/>
@@ -5298,12 +5381,15 @@
       <c r="N101" s="59">
         <v>416</v>
       </c>
-      <c r="O101">
+      <c r="O101" s="95">
         <v>249</v>
       </c>
       <c r="P101" s="2">
         <v>9</v>
       </c>
+      <c r="Q101" s="95"/>
+      <c r="R101" s="95"/>
+      <c r="S101" s="95"/>
       <c r="T101" s="4"/>
     </row>
     <row r="102" spans="1:20" x14ac:dyDescent="0.3">
@@ -5318,20 +5404,20 @@
         <f t="shared" si="6"/>
         <v>414</v>
       </c>
-      <c r="D102" s="60">
+      <c r="D102" s="109">
         <v>384</v>
       </c>
-      <c r="E102" s="3">
+      <c r="E102" s="107">
         <v>203</v>
       </c>
-      <c r="F102" s="29">
+      <c r="F102" s="99">
         <v>8</v>
       </c>
-      <c r="G102" s="32">
+      <c r="G102" s="99">
         <v>21</v>
       </c>
-      <c r="H102" s="30"/>
-      <c r="I102" s="30"/>
+      <c r="H102" s="100"/>
+      <c r="I102" s="100"/>
       <c r="J102" s="31"/>
       <c r="K102" s="30"/>
       <c r="L102" s="29">
@@ -5345,17 +5431,17 @@
       <c r="N102" s="60">
         <v>417</v>
       </c>
-      <c r="O102" s="3">
+      <c r="O102" s="98">
         <v>250</v>
       </c>
       <c r="P102" s="29">
         <v>8</v>
       </c>
-      <c r="Q102" s="32">
+      <c r="Q102" s="99">
         <v>85</v>
       </c>
-      <c r="R102" s="30"/>
-      <c r="S102" s="30"/>
+      <c r="R102" s="100"/>
+      <c r="S102" s="100"/>
       <c r="T102" s="31"/>
     </row>
     <row r="103" spans="1:20" x14ac:dyDescent="0.3">
@@ -5370,20 +5456,20 @@
         <f t="shared" si="6"/>
         <v>416</v>
       </c>
-      <c r="D103" s="75">
+      <c r="D103" s="110">
         <v>385</v>
       </c>
-      <c r="E103" s="73">
+      <c r="E103" s="74">
         <v>204</v>
       </c>
-      <c r="F103" s="81">
+      <c r="F103" s="102">
         <v>47</v>
       </c>
-      <c r="G103" s="79">
+      <c r="G103" s="102">
         <v>95</v>
       </c>
-      <c r="H103" s="73"/>
-      <c r="I103" s="73"/>
+      <c r="H103" s="101"/>
+      <c r="I103" s="101"/>
       <c r="J103" s="85"/>
       <c r="L103" s="35">
         <f t="shared" si="7"/>
@@ -5396,15 +5482,17 @@
       <c r="N103" s="75">
         <v>418</v>
       </c>
-      <c r="O103" s="73">
+      <c r="O103" s="101">
         <v>251</v>
       </c>
       <c r="P103" s="2">
         <v>55</v>
       </c>
-      <c r="Q103" s="79">
+      <c r="Q103" s="102">
         <v>85</v>
       </c>
+      <c r="R103" s="95"/>
+      <c r="S103" s="95"/>
       <c r="T103" s="4"/>
     </row>
     <row r="104" spans="1:20" x14ac:dyDescent="0.3">
@@ -5419,20 +5507,20 @@
         <f t="shared" si="6"/>
         <v>418</v>
       </c>
-      <c r="D104" s="75">
+      <c r="D104" s="110">
         <v>386</v>
       </c>
-      <c r="E104" s="73">
+      <c r="E104" s="74">
         <v>205</v>
       </c>
-      <c r="F104" s="81">
+      <c r="F104" s="102">
         <v>7</v>
       </c>
-      <c r="G104" s="79">
+      <c r="G104" s="102">
         <v>47</v>
       </c>
-      <c r="H104" s="73"/>
-      <c r="I104" s="73"/>
+      <c r="H104" s="101"/>
+      <c r="I104" s="101"/>
       <c r="J104" s="85"/>
       <c r="L104" s="81">
         <f t="shared" si="7"/>
@@ -5445,12 +5533,15 @@
       <c r="N104" s="78">
         <v>419</v>
       </c>
-      <c r="O104" s="73">
+      <c r="O104" s="101">
         <v>252</v>
       </c>
       <c r="P104" s="2">
         <v>7</v>
       </c>
+      <c r="Q104" s="95"/>
+      <c r="R104" s="95"/>
+      <c r="S104" s="95"/>
       <c r="T104" s="4"/>
     </row>
     <row r="105" spans="1:20" x14ac:dyDescent="0.3">
@@ -5465,18 +5556,20 @@
         <f t="shared" si="6"/>
         <v>420</v>
       </c>
-      <c r="D105" s="59">
+      <c r="D105" s="97">
         <v>387</v>
       </c>
-      <c r="E105">
+      <c r="E105" s="25">
         <v>206</v>
       </c>
-      <c r="F105" s="2">
+      <c r="F105" s="98">
         <v>8</v>
       </c>
-      <c r="G105" s="3">
+      <c r="G105" s="98">
         <v>57</v>
       </c>
+      <c r="H105" s="95"/>
+      <c r="I105" s="95"/>
       <c r="J105" s="4"/>
       <c r="L105" s="5">
         <f t="shared" si="7"/>
@@ -5489,12 +5582,15 @@
       <c r="N105" s="59">
         <v>420</v>
       </c>
-      <c r="O105">
+      <c r="O105" s="95">
         <v>253</v>
       </c>
       <c r="P105" s="2">
         <v>8</v>
       </c>
+      <c r="Q105" s="95"/>
+      <c r="R105" s="95"/>
+      <c r="S105" s="95"/>
       <c r="T105" s="4"/>
     </row>
     <row r="106" spans="1:20" x14ac:dyDescent="0.3">
@@ -5509,18 +5605,20 @@
         <f t="shared" si="6"/>
         <v>422</v>
       </c>
-      <c r="D106" s="59">
+      <c r="D106" s="97">
         <v>388</v>
       </c>
-      <c r="E106">
+      <c r="E106" s="25">
         <v>207</v>
       </c>
-      <c r="F106" s="2">
+      <c r="F106" s="98">
         <v>27</v>
       </c>
-      <c r="G106" s="3">
+      <c r="G106" s="98">
         <v>57</v>
       </c>
+      <c r="H106" s="95"/>
+      <c r="I106" s="95"/>
       <c r="J106" s="4"/>
       <c r="L106" s="5">
         <f t="shared" si="7"/>
@@ -5533,12 +5631,15 @@
       <c r="N106" s="59">
         <v>421</v>
       </c>
-      <c r="O106">
+      <c r="O106" s="95">
         <v>254</v>
       </c>
       <c r="P106" s="2">
         <v>39</v>
       </c>
+      <c r="Q106" s="95"/>
+      <c r="R106" s="95"/>
+      <c r="S106" s="95"/>
       <c r="T106" s="4"/>
     </row>
     <row r="107" spans="1:20" x14ac:dyDescent="0.3">
@@ -5553,18 +5654,20 @@
         <f t="shared" si="6"/>
         <v>424</v>
       </c>
-      <c r="D107" s="59">
+      <c r="D107" s="97">
         <v>389</v>
       </c>
-      <c r="E107">
+      <c r="E107" s="25">
         <v>208</v>
       </c>
-      <c r="F107" s="2">
+      <c r="F107" s="98">
         <v>27</v>
       </c>
-      <c r="G107" s="3">
+      <c r="G107" s="98">
         <v>88</v>
       </c>
+      <c r="H107" s="95"/>
+      <c r="I107" s="95"/>
       <c r="J107" s="4"/>
       <c r="L107" s="5">
         <f t="shared" si="7"/>
@@ -5577,12 +5680,15 @@
       <c r="N107" s="59">
         <v>422</v>
       </c>
-      <c r="O107">
+      <c r="O107" s="95">
         <v>255</v>
       </c>
       <c r="P107" s="2">
         <v>55</v>
       </c>
+      <c r="Q107" s="95"/>
+      <c r="R107" s="95"/>
+      <c r="S107" s="95"/>
       <c r="T107" s="4"/>
     </row>
     <row r="108" spans="1:20" x14ac:dyDescent="0.3">
@@ -5597,18 +5703,20 @@
         <f t="shared" si="6"/>
         <v>426</v>
       </c>
-      <c r="D108" s="59">
+      <c r="D108" s="97">
         <v>390</v>
       </c>
-      <c r="E108">
+      <c r="E108" s="25">
         <v>209</v>
       </c>
-      <c r="F108" s="2">
+      <c r="F108" s="98">
         <v>27</v>
       </c>
-      <c r="G108" s="3">
+      <c r="G108" s="98">
         <v>88</v>
       </c>
+      <c r="H108" s="95"/>
+      <c r="I108" s="95"/>
       <c r="J108" s="4"/>
       <c r="L108" s="5">
         <f t="shared" si="7"/>
@@ -5621,12 +5729,15 @@
       <c r="N108" s="59">
         <v>423</v>
       </c>
-      <c r="O108">
+      <c r="O108" s="95">
         <v>256</v>
       </c>
       <c r="P108" s="2">
         <v>55</v>
       </c>
+      <c r="Q108" s="95"/>
+      <c r="R108" s="95"/>
+      <c r="S108" s="95"/>
       <c r="T108" s="4"/>
     </row>
     <row r="109" spans="1:20" x14ac:dyDescent="0.3">
@@ -5641,18 +5752,20 @@
         <f t="shared" si="6"/>
         <v>428</v>
       </c>
-      <c r="D109" s="59">
+      <c r="D109" s="97">
         <v>391</v>
       </c>
-      <c r="E109">
+      <c r="E109" s="25">
         <v>210</v>
       </c>
-      <c r="F109" s="2">
+      <c r="F109" s="98">
         <v>27</v>
       </c>
-      <c r="G109" s="3">
+      <c r="G109" s="98">
         <v>105</v>
       </c>
+      <c r="H109" s="95"/>
+      <c r="I109" s="95"/>
       <c r="J109" s="4"/>
       <c r="L109" s="5">
         <f t="shared" si="7"/>
@@ -5665,12 +5778,15 @@
       <c r="N109" s="59">
         <v>424</v>
       </c>
-      <c r="O109">
+      <c r="O109" s="95">
         <v>257</v>
       </c>
       <c r="P109" s="2">
         <v>55</v>
       </c>
+      <c r="Q109" s="95"/>
+      <c r="R109" s="95"/>
+      <c r="S109" s="95"/>
       <c r="T109" s="4"/>
     </row>
     <row r="110" spans="1:20" x14ac:dyDescent="0.3">
@@ -5685,18 +5801,20 @@
         <f t="shared" si="6"/>
         <v>430</v>
       </c>
-      <c r="D110" s="59">
+      <c r="D110" s="97">
         <v>392</v>
       </c>
-      <c r="E110">
+      <c r="E110" s="25">
         <v>211</v>
       </c>
-      <c r="F110" s="2">
+      <c r="F110" s="98">
         <v>38</v>
       </c>
-      <c r="G110" s="3">
+      <c r="G110" s="98">
         <v>95</v>
       </c>
+      <c r="H110" s="95"/>
+      <c r="I110" s="95"/>
       <c r="J110" s="4"/>
       <c r="L110" s="5">
         <f t="shared" si="7"/>
@@ -5709,12 +5827,15 @@
       <c r="N110" s="59">
         <v>425</v>
       </c>
-      <c r="O110">
+      <c r="O110" s="95">
         <v>258</v>
       </c>
       <c r="P110" s="2">
         <v>38</v>
       </c>
+      <c r="Q110" s="95"/>
+      <c r="R110" s="95"/>
+      <c r="S110" s="95"/>
       <c r="T110" s="4"/>
     </row>
     <row r="111" spans="1:20" x14ac:dyDescent="0.3">
@@ -5729,22 +5850,22 @@
         <f t="shared" si="6"/>
         <v>432</v>
       </c>
-      <c r="D111" s="75">
+      <c r="D111" s="110">
         <v>393</v>
       </c>
-      <c r="E111" s="73">
+      <c r="E111" s="74">
         <v>212</v>
       </c>
-      <c r="F111" s="81">
+      <c r="F111" s="102">
         <v>38</v>
       </c>
-      <c r="G111" s="79">
+      <c r="G111" s="102">
         <v>47</v>
       </c>
-      <c r="H111" s="79">
+      <c r="H111" s="102">
         <v>62</v>
       </c>
-      <c r="I111" s="79">
+      <c r="I111" s="102">
         <v>78</v>
       </c>
       <c r="J111" s="85"/>
@@ -5759,15 +5880,17 @@
       <c r="N111" s="75">
         <v>426</v>
       </c>
-      <c r="O111" s="73">
+      <c r="O111" s="101">
         <v>259</v>
       </c>
       <c r="P111" s="2">
         <v>38</v>
       </c>
-      <c r="Q111" s="79">
+      <c r="Q111" s="102">
         <v>84</v>
       </c>
+      <c r="R111" s="95"/>
+      <c r="S111" s="95"/>
       <c r="T111" s="4"/>
     </row>
     <row r="112" spans="1:20" x14ac:dyDescent="0.3">
@@ -5782,22 +5905,22 @@
         <f t="shared" si="6"/>
         <v>434</v>
       </c>
-      <c r="D112" s="59">
+      <c r="D112" s="97">
         <v>394</v>
       </c>
-      <c r="E112">
+      <c r="E112" s="25">
         <v>213</v>
       </c>
-      <c r="F112" s="2">
+      <c r="F112" s="98">
         <v>9</v>
       </c>
-      <c r="G112" s="3">
+      <c r="G112" s="98">
         <v>47</v>
       </c>
-      <c r="H112" s="3">
+      <c r="H112" s="98">
         <v>62</v>
       </c>
-      <c r="I112" s="3">
+      <c r="I112" s="98">
         <v>78</v>
       </c>
       <c r="J112" s="4"/>
@@ -5812,15 +5935,17 @@
       <c r="N112" s="59">
         <v>427</v>
       </c>
-      <c r="O112">
+      <c r="O112" s="95">
         <v>260</v>
       </c>
       <c r="P112" s="2">
         <v>9</v>
       </c>
-      <c r="Q112" s="3">
+      <c r="Q112" s="98">
         <v>84</v>
       </c>
+      <c r="R112" s="95"/>
+      <c r="S112" s="95"/>
       <c r="T112" s="4"/>
     </row>
     <row r="113" spans="1:20" x14ac:dyDescent="0.3">
@@ -5835,23 +5960,23 @@
         <f t="shared" si="6"/>
         <v>436</v>
       </c>
-      <c r="D113" s="78">
+      <c r="D113" s="111">
         <v>395</v>
       </c>
-      <c r="E113" s="79">
+      <c r="E113" s="77">
         <v>214</v>
       </c>
-      <c r="F113" s="80">
+      <c r="F113" s="103">
         <v>7</v>
       </c>
-      <c r="G113" s="82">
+      <c r="G113" s="103">
         <v>13</v>
       </c>
-      <c r="H113" s="82">
+      <c r="H113" s="103">
         <v>78</v>
       </c>
-      <c r="I113" s="87"/>
-      <c r="J113" s="88"/>
+      <c r="I113" s="104"/>
+      <c r="J113" s="86"/>
       <c r="K113" s="30"/>
       <c r="L113" s="80">
         <f t="shared" si="7"/>
@@ -5864,17 +5989,17 @@
       <c r="N113" s="78">
         <v>428</v>
       </c>
-      <c r="O113" s="79">
+      <c r="O113" s="102">
         <v>261</v>
       </c>
       <c r="P113" s="29">
         <v>7</v>
       </c>
-      <c r="Q113" s="32">
+      <c r="Q113" s="99">
         <v>13</v>
       </c>
-      <c r="R113" s="30"/>
-      <c r="S113" s="30"/>
+      <c r="R113" s="100"/>
+      <c r="S113" s="100"/>
       <c r="T113" s="31"/>
     </row>
     <row r="114" spans="1:20" x14ac:dyDescent="0.3">
@@ -5889,22 +6014,22 @@
         <f t="shared" si="6"/>
         <v>438</v>
       </c>
-      <c r="D114" s="75">
+      <c r="D114" s="110">
         <v>396</v>
       </c>
-      <c r="E114" s="73">
+      <c r="E114" s="74">
         <v>215</v>
       </c>
-      <c r="F114" s="81">
+      <c r="F114" s="102">
         <v>8</v>
       </c>
-      <c r="G114" s="79">
+      <c r="G114" s="102">
         <v>78</v>
       </c>
-      <c r="H114" s="79">
+      <c r="H114" s="102">
         <v>105</v>
       </c>
-      <c r="I114" s="73"/>
+      <c r="I114" s="101"/>
       <c r="J114" s="85"/>
       <c r="L114" s="35">
         <f t="shared" si="7"/>
@@ -5917,13 +6042,15 @@
       <c r="N114" s="75">
         <v>429</v>
       </c>
-      <c r="O114" s="73">
+      <c r="O114" s="101">
         <v>262</v>
       </c>
       <c r="P114" s="2">
         <v>8</v>
       </c>
-      <c r="Q114" s="73"/>
+      <c r="Q114" s="101"/>
+      <c r="R114" s="95"/>
+      <c r="S114" s="95"/>
       <c r="T114" s="4"/>
     </row>
     <row r="115" spans="1:20" x14ac:dyDescent="0.3">
@@ -5938,21 +6065,22 @@
         <f t="shared" si="6"/>
         <v>440</v>
       </c>
-      <c r="D115" s="59">
+      <c r="D115" s="97">
         <v>397</v>
       </c>
-      <c r="E115">
+      <c r="E115" s="25">
         <v>216</v>
       </c>
-      <c r="F115" s="2">
+      <c r="F115" s="98">
         <v>96</v>
       </c>
-      <c r="G115" s="3">
+      <c r="G115" s="98">
         <v>96</v>
       </c>
-      <c r="H115" s="3">
+      <c r="H115" s="98">
         <v>97</v>
       </c>
+      <c r="I115" s="98"/>
       <c r="J115" s="4"/>
       <c r="L115" s="5">
         <f t="shared" si="7"/>
@@ -5965,53 +6093,56 @@
       <c r="N115" s="59">
         <v>430</v>
       </c>
-      <c r="O115">
+      <c r="O115" s="95">
         <v>263</v>
       </c>
       <c r="P115" s="5"/>
+      <c r="Q115" s="95"/>
+      <c r="R115" s="95"/>
+      <c r="S115" s="95"/>
       <c r="T115" s="4"/>
     </row>
     <row r="116" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>4</v>
       </c>
-      <c r="B116" s="6">
-        <f t="shared" si="5"/>
+      <c r="B116" s="5">
+        <f>B115+3</f>
         <v>203</v>
       </c>
-      <c r="C116" s="43">
-        <f t="shared" si="6"/>
+      <c r="C116" s="42">
+        <f>C115+2</f>
         <v>442</v>
       </c>
-      <c r="D116" s="61">
+      <c r="D116" s="97">
         <v>398</v>
       </c>
-      <c r="E116">
+      <c r="E116" s="25">
         <v>217</v>
       </c>
-      <c r="F116" s="69">
+      <c r="F116" s="98">
         <v>96</v>
       </c>
-      <c r="G116" s="18">
+      <c r="G116" s="98">
         <v>96</v>
       </c>
-      <c r="H116" s="18">
+      <c r="H116" s="98">
         <v>97</v>
       </c>
-      <c r="I116" s="7"/>
-      <c r="J116" s="8"/>
+      <c r="I116" s="95"/>
+      <c r="J116" s="4"/>
       <c r="L116" s="6">
-        <f t="shared" si="7"/>
+        <f>L115+3</f>
         <v>203</v>
       </c>
       <c r="M116" s="43">
-        <f t="shared" si="4"/>
+        <f>M115+2</f>
         <v>475</v>
       </c>
       <c r="N116" s="61">
         <v>431</v>
       </c>
-      <c r="O116">
+      <c r="O116" s="7">
         <v>264</v>
       </c>
       <c r="P116" s="6"/>
@@ -6020,338 +6151,247 @@
       <c r="S116" s="7"/>
       <c r="T116" s="8"/>
     </row>
-    <row r="118" spans="1:20" ht="18" x14ac:dyDescent="0.35">
-      <c r="B118" s="14" t="s">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A117">
+        <v>4</v>
+      </c>
+      <c r="B117" s="5">
+        <f>B116+3</f>
+        <v>206</v>
+      </c>
+      <c r="C117" s="42"/>
+      <c r="D117" s="97"/>
+      <c r="E117" s="25">
+        <v>218</v>
+      </c>
+      <c r="F117" s="98">
+        <v>106</v>
+      </c>
+      <c r="G117" s="95"/>
+      <c r="H117" s="95"/>
+      <c r="I117" s="95"/>
+      <c r="J117" s="4"/>
+      <c r="L117" s="95"/>
+      <c r="M117" s="96"/>
+      <c r="N117" s="97"/>
+      <c r="O117" s="95"/>
+      <c r="P117" s="95"/>
+      <c r="Q117" s="95"/>
+      <c r="R117" s="95"/>
+      <c r="S117" s="95"/>
+      <c r="T117" s="95"/>
+    </row>
+    <row r="118" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A118">
+        <v>4</v>
+      </c>
+      <c r="B118" s="6">
+        <f>B117+3</f>
+        <v>209</v>
+      </c>
+      <c r="C118" s="43"/>
+      <c r="D118" s="105"/>
+      <c r="E118" s="34">
+        <v>219</v>
+      </c>
+      <c r="F118" s="18">
+        <v>106</v>
+      </c>
+      <c r="G118" s="7"/>
+      <c r="H118" s="7"/>
+      <c r="I118" s="7"/>
+      <c r="J118" s="8"/>
+      <c r="L118" s="95"/>
+      <c r="M118" s="96"/>
+      <c r="N118" s="97"/>
+      <c r="O118" s="95"/>
+      <c r="P118" s="95"/>
+      <c r="Q118" s="95"/>
+      <c r="R118" s="95"/>
+      <c r="S118" s="95"/>
+      <c r="T118" s="95"/>
+    </row>
+    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="C119" s="89"/>
+      <c r="D119" s="90"/>
+      <c r="M119" s="89"/>
+      <c r="N119" s="90"/>
+    </row>
+    <row r="121" spans="1:20" ht="18" x14ac:dyDescent="0.35">
+      <c r="B121" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C118" s="14" t="s">
+      <c r="C121" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="D118" s="14"/>
-      <c r="E118" s="1"/>
-      <c r="F118" s="1"/>
-      <c r="G118" s="1"/>
-    </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B119" s="1"/>
-      <c r="C119" s="1"/>
-      <c r="D119" s="1"/>
-      <c r="E119" s="11"/>
-      <c r="F119" s="1"/>
-      <c r="G119" s="1"/>
-    </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B120" s="9" t="s">
+      <c r="D121" s="14"/>
+      <c r="E121" s="1"/>
+      <c r="F121" s="1"/>
+      <c r="G121" s="1"/>
+    </row>
+    <row r="122" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B122" s="1"/>
+      <c r="C122" s="1"/>
+      <c r="D122" s="1"/>
+      <c r="E122" s="11"/>
+      <c r="F122" s="1"/>
+      <c r="G122" s="1"/>
+    </row>
+    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B123" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C120" s="40"/>
-      <c r="D120" s="9"/>
-      <c r="F120" s="93" t="s">
+      <c r="C123" s="40"/>
+      <c r="D123" s="9"/>
+      <c r="F123" s="93" t="s">
         <v>5</v>
       </c>
-      <c r="G120" s="94"/>
-      <c r="H120" s="94"/>
-      <c r="I120" s="94"/>
-      <c r="J120" s="94"/>
-      <c r="L120" s="9" t="s">
+      <c r="G123" s="94"/>
+      <c r="H123" s="94"/>
+      <c r="I123" s="94"/>
+      <c r="J123" s="94"/>
+      <c r="L123" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="M120" s="40"/>
-      <c r="N120" s="9"/>
-      <c r="O120" s="33"/>
-      <c r="P120" s="93" t="s">
+      <c r="M123" s="40"/>
+      <c r="N123" s="9"/>
+      <c r="O123" s="33"/>
+      <c r="P123" s="93" t="s">
         <v>5</v>
       </c>
-      <c r="Q120" s="94"/>
-      <c r="R120" s="94"/>
-      <c r="S120" s="94"/>
-      <c r="T120" s="94"/>
-    </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B121" s="9" t="s">
+      <c r="Q123" s="94"/>
+      <c r="R123" s="94"/>
+      <c r="S123" s="94"/>
+      <c r="T123" s="94"/>
+    </row>
+    <row r="124" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B124" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C121" s="45" t="s">
+      <c r="C124" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="D121" s="63" t="s">
+      <c r="D124" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="E121" s="13" t="s">
+      <c r="E124" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="F121" s="10" t="s">
+      <c r="F124" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G121" s="11" t="s">
+      <c r="G124" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="H121" s="11" t="s">
+      <c r="H124" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="I121" s="11" t="s">
+      <c r="I124" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J121" s="12" t="s">
+      <c r="J124" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="L121" s="9" t="s">
+      <c r="L124" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="M121" s="40" t="s">
+      <c r="M124" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="N121" s="57" t="s">
+      <c r="N124" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="O121" s="13" t="s">
+      <c r="O124" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="P121" s="10" t="s">
+      <c r="P124" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="Q121" s="11" t="s">
+      <c r="Q124" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="R121" s="11" t="s">
+      <c r="R124" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="S121" s="11" t="s">
+      <c r="S124" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="T121" s="12" t="s">
+      <c r="T124" s="12" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A122">
-        <v>8</v>
-      </c>
-      <c r="B122">
-        <v>110</v>
-      </c>
-      <c r="C122" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="D122" s="52">
-        <v>402</v>
-      </c>
-      <c r="E122">
-        <v>220</v>
-      </c>
-      <c r="F122" s="2">
-        <v>94</v>
-      </c>
-      <c r="J122" s="4"/>
-      <c r="K122" s="30"/>
-      <c r="L122" s="5">
-        <v>110</v>
-      </c>
-      <c r="M122" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="N122" s="59">
-        <v>435</v>
-      </c>
-      <c r="O122">
-        <v>267</v>
-      </c>
-      <c r="P122" s="28"/>
-      <c r="Q122" s="30"/>
-      <c r="R122" s="30"/>
-      <c r="S122" s="30"/>
-      <c r="T122" s="31"/>
-    </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A123">
-        <v>8</v>
-      </c>
-      <c r="B123">
-        <v>116</v>
-      </c>
-      <c r="C123" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="D123" s="52">
-        <v>403</v>
-      </c>
-      <c r="E123">
-        <v>221</v>
-      </c>
-      <c r="F123" s="2">
-        <v>94</v>
-      </c>
-      <c r="J123" s="4"/>
-      <c r="L123" s="5">
-        <v>116</v>
-      </c>
-      <c r="M123" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="N123" s="59">
-        <v>436</v>
-      </c>
-      <c r="O123">
-        <v>268</v>
-      </c>
-      <c r="P123" s="3">
-        <v>52</v>
-      </c>
-      <c r="T123" s="4"/>
-    </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A124">
-        <v>8</v>
-      </c>
-      <c r="B124" s="32">
-        <v>122</v>
-      </c>
-      <c r="C124" s="56" t="s">
-        <v>25</v>
-      </c>
-      <c r="D124" s="53">
-        <v>404</v>
-      </c>
-      <c r="E124" s="3">
-        <v>222</v>
-      </c>
-      <c r="F124" s="29">
-        <v>10</v>
-      </c>
-      <c r="G124" s="32">
-        <v>12</v>
-      </c>
-      <c r="H124" s="32">
-        <v>37</v>
-      </c>
-      <c r="I124" s="32">
-        <v>76</v>
-      </c>
-      <c r="J124" s="31"/>
-      <c r="L124" s="29">
-        <v>122</v>
-      </c>
-      <c r="M124" s="56" t="s">
-        <v>25</v>
-      </c>
-      <c r="N124" s="60">
-        <v>437</v>
-      </c>
-      <c r="O124" s="3">
-        <v>269</v>
-      </c>
-      <c r="P124" s="29">
-        <v>11</v>
-      </c>
-      <c r="Q124" s="32">
-        <v>16</v>
-      </c>
-      <c r="R124" s="3">
-        <v>52</v>
-      </c>
-      <c r="S124" s="30"/>
-      <c r="T124" s="31"/>
     </row>
     <row r="125" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>8</v>
       </c>
-      <c r="B125" s="73">
-        <v>128</v>
-      </c>
-      <c r="C125" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="D125" s="74">
-        <v>405</v>
-      </c>
-      <c r="E125" s="73">
-        <v>223</v>
-      </c>
-      <c r="F125" s="81">
-        <v>14</v>
-      </c>
-      <c r="G125" s="79">
-        <v>32</v>
-      </c>
-      <c r="H125" s="79">
-        <v>52</v>
-      </c>
-      <c r="I125" s="79">
-        <v>76</v>
-      </c>
-      <c r="J125" s="85"/>
-      <c r="L125" s="35">
-        <v>128</v>
-      </c>
-      <c r="M125" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="N125" s="75">
-        <v>438</v>
-      </c>
-      <c r="O125" s="73">
-        <v>270</v>
-      </c>
-      <c r="P125" s="2">
-        <v>17</v>
-      </c>
-      <c r="Q125" s="3">
-        <v>33</v>
-      </c>
-      <c r="R125" s="3">
-        <v>52</v>
-      </c>
-      <c r="T125" s="4"/>
+      <c r="B125">
+        <v>110</v>
+      </c>
+      <c r="C125" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="D125" s="52">
+        <v>402</v>
+      </c>
+      <c r="E125">
+        <v>220</v>
+      </c>
+      <c r="F125" s="2">
+        <v>94</v>
+      </c>
+      <c r="J125" s="4"/>
+      <c r="K125" s="30"/>
+      <c r="L125" s="5">
+        <v>110</v>
+      </c>
+      <c r="M125" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="N125" s="59">
+        <v>435</v>
+      </c>
+      <c r="O125">
+        <v>267</v>
+      </c>
+      <c r="P125" s="28"/>
+      <c r="Q125" s="30"/>
+      <c r="R125" s="30"/>
+      <c r="S125" s="30"/>
+      <c r="T125" s="31"/>
     </row>
     <row r="126" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>8</v>
       </c>
       <c r="B126">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="C126" s="46" t="s">
         <v>25</v>
       </c>
       <c r="D126" s="52">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="E126">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="F126" s="2">
-        <v>14</v>
-      </c>
-      <c r="G126" s="3">
-        <v>32</v>
-      </c>
-      <c r="H126" s="3">
-        <v>52</v>
-      </c>
-      <c r="I126" s="3">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="J126" s="4"/>
       <c r="L126" s="5">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="M126" s="46" t="s">
         <v>25</v>
       </c>
       <c r="N126" s="59">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="O126">
-        <v>271</v>
-      </c>
-      <c r="P126" s="2">
-        <v>17</v>
-      </c>
-      <c r="Q126" s="3">
-        <v>37</v>
-      </c>
-      <c r="R126" s="3">
+        <v>268</v>
+      </c>
+      <c r="P126" s="3">
         <v>52</v>
       </c>
       <c r="T126" s="4"/>
@@ -6360,43 +6400,42 @@
       <c r="A127">
         <v>8</v>
       </c>
-      <c r="B127" s="82">
-        <v>140</v>
-      </c>
-      <c r="C127" s="81" t="s">
-        <v>25</v>
-      </c>
-      <c r="D127" s="77">
-        <v>407</v>
-      </c>
-      <c r="E127" s="79">
-        <v>225</v>
-      </c>
-      <c r="F127" s="80">
+      <c r="B127" s="32">
+        <v>122</v>
+      </c>
+      <c r="C127" s="56" t="s">
+        <v>25</v>
+      </c>
+      <c r="D127" s="53">
+        <v>404</v>
+      </c>
+      <c r="E127" s="3">
+        <v>222</v>
+      </c>
+      <c r="F127" s="29">
         <v>10</v>
       </c>
-      <c r="G127" s="82">
+      <c r="G127" s="32">
         <v>12</v>
       </c>
-      <c r="H127" s="82">
-        <v>53</v>
-      </c>
-      <c r="I127" s="82">
+      <c r="H127" s="32">
+        <v>37</v>
+      </c>
+      <c r="I127" s="32">
         <v>76</v>
       </c>
-      <c r="J127" s="88"/>
-      <c r="K127" s="30"/>
-      <c r="L127" s="80">
-        <v>140</v>
-      </c>
-      <c r="M127" s="81" t="s">
-        <v>25</v>
-      </c>
-      <c r="N127" s="78">
-        <v>440</v>
-      </c>
-      <c r="O127" s="79">
-        <v>272</v>
+      <c r="J127" s="31"/>
+      <c r="L127" s="29">
+        <v>122</v>
+      </c>
+      <c r="M127" s="56" t="s">
+        <v>25</v>
+      </c>
+      <c r="N127" s="60">
+        <v>437</v>
+      </c>
+      <c r="O127" s="3">
+        <v>269</v>
       </c>
       <c r="P127" s="29">
         <v>11</v>
@@ -6414,156 +6453,156 @@
       <c r="A128">
         <v>8</v>
       </c>
-      <c r="B128" s="82">
-        <v>146</v>
-      </c>
-      <c r="C128" s="81" t="s">
-        <v>25</v>
-      </c>
-      <c r="D128" s="77">
-        <v>408</v>
-      </c>
-      <c r="E128" s="79">
-        <v>226</v>
-      </c>
-      <c r="F128" s="80">
+      <c r="B128" s="73">
+        <v>128</v>
+      </c>
+      <c r="C128" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D128" s="74">
+        <v>405</v>
+      </c>
+      <c r="E128" s="73">
+        <v>223</v>
+      </c>
+      <c r="F128" s="81">
         <v>14</v>
       </c>
-      <c r="G128" s="82">
-        <v>23</v>
-      </c>
-      <c r="H128" s="82">
-        <v>53</v>
-      </c>
-      <c r="I128" s="82">
+      <c r="G128" s="79">
+        <v>32</v>
+      </c>
+      <c r="H128" s="79">
+        <v>52</v>
+      </c>
+      <c r="I128" s="79">
         <v>76</v>
       </c>
-      <c r="J128" s="88"/>
-      <c r="L128" s="80">
-        <v>146</v>
-      </c>
-      <c r="M128" s="81" t="s">
-        <v>25</v>
-      </c>
-      <c r="N128" s="78">
-        <v>441</v>
-      </c>
-      <c r="O128" s="79">
-        <v>273</v>
-      </c>
-      <c r="P128" s="29">
+      <c r="J128" s="85"/>
+      <c r="L128" s="35">
+        <v>128</v>
+      </c>
+      <c r="M128" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="N128" s="75">
+        <v>438</v>
+      </c>
+      <c r="O128" s="73">
+        <v>270</v>
+      </c>
+      <c r="P128" s="2">
         <v>17</v>
       </c>
-      <c r="Q128" s="32">
-        <v>29</v>
+      <c r="Q128" s="3">
+        <v>33</v>
       </c>
       <c r="R128" s="3">
         <v>52</v>
       </c>
-      <c r="S128" s="30"/>
-      <c r="T128" s="31"/>
+      <c r="T128" s="4"/>
     </row>
     <row r="129" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>8</v>
       </c>
       <c r="B129">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="C129" s="46" t="s">
         <v>25</v>
       </c>
       <c r="D129" s="52">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="E129">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F129" s="2">
         <v>14</v>
       </c>
-      <c r="G129" s="32">
-        <v>33</v>
+      <c r="G129" s="3">
+        <v>32</v>
       </c>
       <c r="H129" s="3">
-        <v>51</v>
-      </c>
-      <c r="I129" s="32">
+        <v>52</v>
+      </c>
+      <c r="I129" s="3">
         <v>76</v>
       </c>
       <c r="J129" s="4"/>
-      <c r="K129" s="30"/>
       <c r="L129" s="5">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="M129" s="46" t="s">
         <v>25</v>
       </c>
       <c r="N129" s="59">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="O129">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="P129" s="2">
         <v>17</v>
       </c>
-      <c r="Q129" s="32">
-        <v>29</v>
+      <c r="Q129" s="3">
+        <v>37</v>
       </c>
       <c r="R129" s="3">
-        <v>53</v>
-      </c>
-      <c r="S129" s="30"/>
-      <c r="T129" s="31"/>
+        <v>52</v>
+      </c>
+      <c r="T129" s="4"/>
     </row>
     <row r="130" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>8</v>
       </c>
-      <c r="B130" s="32">
-        <v>158</v>
-      </c>
-      <c r="C130" s="56" t="s">
-        <v>25</v>
-      </c>
-      <c r="D130" s="53">
-        <v>410</v>
-      </c>
-      <c r="E130" s="3">
-        <v>228</v>
-      </c>
-      <c r="F130" s="29">
+      <c r="B130" s="82">
+        <v>140</v>
+      </c>
+      <c r="C130" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="D130" s="77">
+        <v>407</v>
+      </c>
+      <c r="E130" s="79">
+        <v>225</v>
+      </c>
+      <c r="F130" s="80">
         <v>10</v>
       </c>
-      <c r="G130" s="32">
+      <c r="G130" s="82">
         <v>12</v>
       </c>
-      <c r="H130" s="32">
-        <v>51</v>
-      </c>
-      <c r="I130" s="30"/>
-      <c r="J130" s="31"/>
-      <c r="L130" s="29">
-        <v>158</v>
-      </c>
-      <c r="M130" s="56" t="s">
-        <v>25</v>
-      </c>
-      <c r="N130" s="60">
-        <v>443</v>
-      </c>
-      <c r="O130" s="3">
-        <v>275</v>
+      <c r="H130" s="82">
+        <v>53</v>
+      </c>
+      <c r="I130" s="82">
+        <v>76</v>
+      </c>
+      <c r="J130" s="86"/>
+      <c r="K130" s="30"/>
+      <c r="L130" s="80">
+        <v>140</v>
+      </c>
+      <c r="M130" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="N130" s="78">
+        <v>440</v>
+      </c>
+      <c r="O130" s="79">
+        <v>272</v>
       </c>
       <c r="P130" s="29">
         <v>11</v>
       </c>
       <c r="Q130" s="32">
-        <v>29</v>
-      </c>
-      <c r="R130" s="32">
-        <v>53</v>
+        <v>16</v>
+      </c>
+      <c r="R130" s="3">
+        <v>52</v>
       </c>
       <c r="S130" s="30"/>
       <c r="T130" s="31"/>
@@ -6572,208 +6611,209 @@
       <c r="A131">
         <v>8</v>
       </c>
-      <c r="B131" s="73">
-        <v>164</v>
-      </c>
-      <c r="C131" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="D131" s="74">
-        <v>411</v>
-      </c>
-      <c r="E131" s="73">
-        <v>229</v>
-      </c>
-      <c r="F131" s="81">
-        <v>18</v>
-      </c>
-      <c r="G131" s="79">
-        <v>28</v>
-      </c>
-      <c r="H131" s="79">
-        <v>51</v>
-      </c>
-      <c r="I131" s="79">
-        <v>66</v>
-      </c>
-      <c r="J131" s="85"/>
-      <c r="L131" s="35">
-        <v>164</v>
-      </c>
-      <c r="M131" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="N131" s="75">
-        <v>444</v>
-      </c>
-      <c r="O131" s="73">
-        <v>276</v>
-      </c>
-      <c r="P131" s="2">
+      <c r="B131" s="82">
+        <v>146</v>
+      </c>
+      <c r="C131" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="D131" s="77">
+        <v>408</v>
+      </c>
+      <c r="E131" s="79">
+        <v>226</v>
+      </c>
+      <c r="F131" s="80">
         <v>14</v>
+      </c>
+      <c r="G131" s="82">
+        <v>23</v>
+      </c>
+      <c r="H131" s="82">
+        <v>53</v>
+      </c>
+      <c r="I131" s="82">
+        <v>76</v>
+      </c>
+      <c r="J131" s="86"/>
+      <c r="L131" s="80">
+        <v>146</v>
+      </c>
+      <c r="M131" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="N131" s="78">
+        <v>441</v>
+      </c>
+      <c r="O131" s="79">
+        <v>273</v>
+      </c>
+      <c r="P131" s="29">
+        <v>17</v>
       </c>
       <c r="Q131" s="32">
         <v>29</v>
       </c>
       <c r="R131" s="3">
-        <v>53</v>
-      </c>
-      <c r="T131" s="4"/>
+        <v>52</v>
+      </c>
+      <c r="S131" s="30"/>
+      <c r="T131" s="31"/>
     </row>
     <row r="132" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>8</v>
       </c>
       <c r="B132">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="C132" s="46" t="s">
         <v>25</v>
       </c>
       <c r="D132" s="52">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="E132">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F132" s="2">
-        <v>18</v>
-      </c>
-      <c r="G132" s="3">
-        <v>28</v>
+        <v>14</v>
+      </c>
+      <c r="G132" s="32">
+        <v>33</v>
       </c>
       <c r="H132" s="3">
         <v>51</v>
       </c>
-      <c r="I132" s="3">
-        <v>66</v>
+      <c r="I132" s="32">
+        <v>76</v>
       </c>
       <c r="J132" s="4"/>
+      <c r="K132" s="30"/>
       <c r="L132" s="5">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="M132" s="46" t="s">
         <v>25</v>
       </c>
       <c r="N132" s="59">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="O132">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="P132" s="2">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="Q132" s="32">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="R132" s="3">
         <v>53</v>
       </c>
-      <c r="T132" s="4"/>
+      <c r="S132" s="30"/>
+      <c r="T132" s="31"/>
     </row>
     <row r="133" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>8</v>
       </c>
-      <c r="B133">
-        <v>176</v>
-      </c>
-      <c r="C133" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="D133" s="52">
-        <v>413</v>
-      </c>
-      <c r="E133">
-        <v>231</v>
-      </c>
-      <c r="F133" s="2">
-        <v>18</v>
-      </c>
-      <c r="G133" s="3">
-        <v>28</v>
-      </c>
-      <c r="H133" s="3">
-        <v>41</v>
-      </c>
-      <c r="I133" s="3">
-        <v>59</v>
-      </c>
-      <c r="J133" s="4"/>
-      <c r="L133" s="5">
-        <v>176</v>
-      </c>
-      <c r="M133" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="N133" s="59">
-        <v>446</v>
-      </c>
-      <c r="O133">
-        <v>278</v>
-      </c>
-      <c r="P133" s="2">
-        <v>19</v>
+      <c r="B133" s="32">
+        <v>158</v>
+      </c>
+      <c r="C133" s="56" t="s">
+        <v>25</v>
+      </c>
+      <c r="D133" s="53">
+        <v>410</v>
+      </c>
+      <c r="E133" s="3">
+        <v>228</v>
+      </c>
+      <c r="F133" s="29">
+        <v>10</v>
+      </c>
+      <c r="G133" s="32">
+        <v>12</v>
+      </c>
+      <c r="H133" s="32">
+        <v>51</v>
+      </c>
+      <c r="I133" s="30"/>
+      <c r="J133" s="31"/>
+      <c r="L133" s="29">
+        <v>158</v>
+      </c>
+      <c r="M133" s="56" t="s">
+        <v>25</v>
+      </c>
+      <c r="N133" s="60">
+        <v>443</v>
+      </c>
+      <c r="O133" s="3">
+        <v>275</v>
+      </c>
+      <c r="P133" s="29">
+        <v>11</v>
       </c>
       <c r="Q133" s="32">
-        <v>31</v>
-      </c>
-      <c r="R133" s="3">
-        <v>41</v>
-      </c>
-      <c r="T133" s="4"/>
+        <v>29</v>
+      </c>
+      <c r="R133" s="32">
+        <v>53</v>
+      </c>
+      <c r="S133" s="30"/>
+      <c r="T133" s="31"/>
     </row>
     <row r="134" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>8</v>
       </c>
-      <c r="B134">
-        <v>182</v>
-      </c>
-      <c r="C134" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="D134" s="52">
-        <v>414</v>
-      </c>
-      <c r="E134">
-        <v>232</v>
-      </c>
-      <c r="F134" s="2">
+      <c r="B134" s="73">
+        <v>164</v>
+      </c>
+      <c r="C134" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D134" s="74">
+        <v>411</v>
+      </c>
+      <c r="E134" s="73">
+        <v>229</v>
+      </c>
+      <c r="F134" s="81">
         <v>18</v>
       </c>
-      <c r="G134" s="3">
+      <c r="G134" s="79">
         <v>28</v>
       </c>
-      <c r="H134" s="3">
-        <v>42</v>
-      </c>
-      <c r="I134" s="3">
-        <v>59</v>
-      </c>
-      <c r="J134" s="4"/>
-      <c r="K134" s="30"/>
-      <c r="L134" s="5">
-        <v>182</v>
-      </c>
-      <c r="M134" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="N134" s="59">
-        <v>447</v>
-      </c>
-      <c r="O134">
-        <v>279</v>
+      <c r="H134" s="79">
+        <v>51</v>
+      </c>
+      <c r="I134" s="79">
+        <v>66</v>
+      </c>
+      <c r="J134" s="85"/>
+      <c r="L134" s="35">
+        <v>164</v>
+      </c>
+      <c r="M134" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="N134" s="75">
+        <v>444</v>
+      </c>
+      <c r="O134" s="73">
+        <v>276</v>
       </c>
       <c r="P134" s="2">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="Q134" s="32">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="R134" s="3">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="T134" s="4"/>
     </row>
@@ -6781,53 +6821,51 @@
       <c r="A135">
         <v>8</v>
       </c>
-      <c r="B135" s="73">
-        <v>188</v>
-      </c>
-      <c r="C135" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="D135" s="74">
-        <v>415</v>
-      </c>
-      <c r="E135" s="73">
-        <v>233</v>
-      </c>
-      <c r="F135" s="81">
-        <v>33</v>
-      </c>
-      <c r="G135" s="79">
-        <v>37</v>
-      </c>
-      <c r="H135" s="79">
-        <v>41</v>
-      </c>
-      <c r="I135" s="79">
-        <v>59</v>
-      </c>
-      <c r="J135" s="89">
-        <v>75</v>
-      </c>
-      <c r="L135" s="35">
-        <v>188</v>
-      </c>
-      <c r="M135" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="N135" s="75">
-        <v>448</v>
-      </c>
-      <c r="O135" s="73">
-        <v>280</v>
+      <c r="B135">
+        <v>170</v>
+      </c>
+      <c r="C135" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="D135" s="52">
+        <v>412</v>
+      </c>
+      <c r="E135">
+        <v>230</v>
+      </c>
+      <c r="F135" s="2">
+        <v>18</v>
+      </c>
+      <c r="G135" s="3">
+        <v>28</v>
+      </c>
+      <c r="H135" s="3">
+        <v>51</v>
+      </c>
+      <c r="I135" s="3">
+        <v>66</v>
+      </c>
+      <c r="J135" s="4"/>
+      <c r="L135" s="5">
+        <v>170</v>
+      </c>
+      <c r="M135" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="N135" s="59">
+        <v>445</v>
+      </c>
+      <c r="O135">
+        <v>277</v>
       </c>
       <c r="P135" s="2">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="Q135" s="32">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="R135" s="3">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="T135" s="4"/>
     </row>
@@ -6835,198 +6873,357 @@
       <c r="A136">
         <v>8</v>
       </c>
-      <c r="B136" s="82">
-        <v>194</v>
-      </c>
-      <c r="C136" s="81" t="s">
-        <v>25</v>
-      </c>
-      <c r="D136" s="77">
-        <v>416</v>
-      </c>
-      <c r="E136" s="79">
-        <v>234</v>
-      </c>
-      <c r="F136" s="80">
-        <v>10</v>
-      </c>
-      <c r="G136" s="82">
-        <v>12</v>
-      </c>
-      <c r="H136" s="82">
-        <v>42</v>
-      </c>
-      <c r="I136" s="82">
+      <c r="B136">
+        <v>176</v>
+      </c>
+      <c r="C136" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="D136" s="52">
+        <v>413</v>
+      </c>
+      <c r="E136">
+        <v>231</v>
+      </c>
+      <c r="F136" s="2">
+        <v>18</v>
+      </c>
+      <c r="G136" s="3">
+        <v>28</v>
+      </c>
+      <c r="H136" s="3">
+        <v>41</v>
+      </c>
+      <c r="I136" s="3">
         <v>59</v>
       </c>
-      <c r="J136" s="90">
-        <v>75</v>
-      </c>
-      <c r="L136" s="80">
-        <v>194</v>
-      </c>
-      <c r="M136" s="81" t="s">
-        <v>25</v>
-      </c>
-      <c r="N136" s="78">
-        <v>449</v>
-      </c>
-      <c r="O136" s="79">
-        <v>281</v>
-      </c>
-      <c r="P136" s="29">
-        <v>11</v>
+      <c r="J136" s="4"/>
+      <c r="L136" s="5">
+        <v>176</v>
+      </c>
+      <c r="M136" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="N136" s="59">
+        <v>446</v>
+      </c>
+      <c r="O136">
+        <v>278</v>
+      </c>
+      <c r="P136" s="2">
+        <v>19</v>
       </c>
       <c r="Q136" s="32">
         <v>31</v>
       </c>
-      <c r="R136" s="32">
-        <v>42</v>
-      </c>
-      <c r="S136" s="30"/>
-      <c r="T136" s="31"/>
+      <c r="R136" s="3">
+        <v>41</v>
+      </c>
+      <c r="T136" s="4"/>
     </row>
     <row r="137" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>8</v>
       </c>
       <c r="B137">
-        <v>200</v>
+        <v>182</v>
       </c>
       <c r="C137" s="46" t="s">
         <v>25</v>
       </c>
       <c r="D137" s="52">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="E137">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="F137" s="2">
-        <v>98</v>
+        <v>18</v>
       </c>
       <c r="G137" s="3">
-        <v>101</v>
+        <v>28</v>
+      </c>
+      <c r="H137" s="3">
+        <v>42</v>
+      </c>
+      <c r="I137" s="3">
+        <v>59</v>
       </c>
       <c r="J137" s="4"/>
+      <c r="K137" s="30"/>
       <c r="L137" s="5">
-        <v>200</v>
+        <v>182</v>
       </c>
       <c r="M137" s="46" t="s">
         <v>25</v>
       </c>
       <c r="N137" s="59">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="O137">
-        <v>282</v>
-      </c>
-      <c r="P137" s="5"/>
+        <v>279</v>
+      </c>
+      <c r="P137" s="2">
+        <v>19</v>
+      </c>
+      <c r="Q137" s="32">
+        <v>31</v>
+      </c>
+      <c r="R137" s="3">
+        <v>42</v>
+      </c>
       <c r="T137" s="4"/>
     </row>
     <row r="138" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>8</v>
       </c>
-      <c r="B138" s="7">
+      <c r="B138" s="73">
+        <v>188</v>
+      </c>
+      <c r="C138" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D138" s="74">
+        <v>415</v>
+      </c>
+      <c r="E138" s="73">
+        <v>233</v>
+      </c>
+      <c r="F138" s="81">
+        <v>33</v>
+      </c>
+      <c r="G138" s="79">
+        <v>37</v>
+      </c>
+      <c r="H138" s="79">
+        <v>41</v>
+      </c>
+      <c r="I138" s="79">
+        <v>59</v>
+      </c>
+      <c r="J138" s="87">
+        <v>75</v>
+      </c>
+      <c r="L138" s="35">
+        <v>188</v>
+      </c>
+      <c r="M138" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="N138" s="75">
+        <v>448</v>
+      </c>
+      <c r="O138" s="73">
+        <v>280</v>
+      </c>
+      <c r="P138" s="2">
+        <v>33</v>
+      </c>
+      <c r="Q138" s="32">
+        <v>37</v>
+      </c>
+      <c r="R138" s="3">
+        <v>41</v>
+      </c>
+      <c r="T138" s="4"/>
+    </row>
+    <row r="139" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A139">
+        <v>8</v>
+      </c>
+      <c r="B139" s="82">
+        <v>194</v>
+      </c>
+      <c r="C139" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="D139" s="77">
+        <v>416</v>
+      </c>
+      <c r="E139" s="79">
+        <v>234</v>
+      </c>
+      <c r="F139" s="80">
+        <v>10</v>
+      </c>
+      <c r="G139" s="82">
+        <v>12</v>
+      </c>
+      <c r="H139" s="82">
+        <v>42</v>
+      </c>
+      <c r="I139" s="82">
+        <v>59</v>
+      </c>
+      <c r="J139" s="88">
+        <v>75</v>
+      </c>
+      <c r="L139" s="80">
+        <v>194</v>
+      </c>
+      <c r="M139" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="N139" s="78">
+        <v>449</v>
+      </c>
+      <c r="O139" s="79">
+        <v>281</v>
+      </c>
+      <c r="P139" s="29">
+        <v>11</v>
+      </c>
+      <c r="Q139" s="32">
+        <v>31</v>
+      </c>
+      <c r="R139" s="32">
+        <v>42</v>
+      </c>
+      <c r="S139" s="30"/>
+      <c r="T139" s="31"/>
+    </row>
+    <row r="140" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A140">
+        <v>8</v>
+      </c>
+      <c r="B140">
+        <v>200</v>
+      </c>
+      <c r="C140" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="D140" s="52">
+        <v>417</v>
+      </c>
+      <c r="E140">
+        <v>235</v>
+      </c>
+      <c r="F140" s="2">
+        <v>98</v>
+      </c>
+      <c r="G140" s="3">
+        <v>101</v>
+      </c>
+      <c r="J140" s="4"/>
+      <c r="L140" s="5">
+        <v>200</v>
+      </c>
+      <c r="M140" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="N140" s="59">
+        <v>450</v>
+      </c>
+      <c r="O140">
+        <v>282</v>
+      </c>
+      <c r="P140" s="5"/>
+      <c r="T140" s="4"/>
+    </row>
+    <row r="141" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A141">
+        <v>8</v>
+      </c>
+      <c r="B141" s="7">
         <v>206</v>
       </c>
-      <c r="C138" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="D138" s="54">
+      <c r="C141" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="D141" s="54">
         <v>418</v>
       </c>
-      <c r="E138">
+      <c r="E141">
         <v>236</v>
       </c>
-      <c r="F138" s="69">
+      <c r="F141" s="69">
         <v>98</v>
       </c>
-      <c r="G138" s="18">
+      <c r="G141" s="18">
         <v>101</v>
       </c>
-      <c r="H138" s="7"/>
-      <c r="I138" s="7"/>
-      <c r="J138" s="8"/>
-      <c r="L138" s="6">
+      <c r="H141" s="7"/>
+      <c r="I141" s="7"/>
+      <c r="J141" s="8"/>
+      <c r="L141" s="6">
         <v>206</v>
       </c>
-      <c r="M138" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="N138" s="61">
+      <c r="M141" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="N141" s="61">
         <v>451</v>
       </c>
-      <c r="O138">
+      <c r="O141">
         <v>283</v>
       </c>
-      <c r="P138" s="6"/>
-      <c r="Q138" s="7"/>
-      <c r="R138" s="7"/>
-      <c r="S138" s="7"/>
-      <c r="T138" s="8"/>
-    </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B141" t="s">
+      <c r="P141" s="6"/>
+      <c r="Q141" s="7"/>
+      <c r="R141" s="7"/>
+      <c r="S141" s="7"/>
+      <c r="T141" s="8"/>
+    </row>
+    <row r="144" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B144" t="s">
         <v>40</v>
       </c>
-      <c r="C141" t="s">
+      <c r="C144" t="s">
         <v>44</v>
       </c>
-      <c r="D141" t="s">
+      <c r="D144" t="s">
         <v>43</v>
       </c>
-      <c r="L141" t="s">
+      <c r="L144" t="s">
         <v>2</v>
       </c>
-      <c r="M141" t="s">
+      <c r="M144" t="s">
         <v>45</v>
       </c>
-      <c r="N141" t="s">
+      <c r="N144" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="142" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B142" t="s">
+    <row r="145" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B145" t="s">
         <v>41</v>
       </c>
-      <c r="L142" t="s">
+      <c r="L145" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="143" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B143">
+    <row r="146" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B146">
         <v>125</v>
       </c>
-      <c r="L143">
+      <c r="L146">
         <v>127</v>
       </c>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B144">
+    <row r="147" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B147">
         <v>126</v>
       </c>
-      <c r="L144">
+      <c r="L147">
         <v>128</v>
       </c>
     </row>
-    <row r="146" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B146" t="s">
+    <row r="149" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B149" t="s">
         <v>42</v>
       </c>
-      <c r="L146" t="s">
+      <c r="L149" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="147" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B147" t="str">
-        <f ca="1">"3,1,"&amp;INDIRECT(D141&amp;B143)&amp;","&amp;INDIRECT(D141&amp;B144)&amp;",0,-1,NONE,NONE,SO MINISCAN "&amp;A138&amp;"KHZ STARTING ORDER "&amp;INDIRECT(C141&amp;B143)&amp;" &amp; "&amp;INDIRECT(C141&amp;B144)</f>
-        <v>3,1,223,224,0,-1,NONE,NONE,SO MINISCAN 8KHZ STARTING ORDER 128 &amp; 134</v>
-      </c>
-      <c r="L147" t="str">
-        <f ca="1">"3,1,"&amp;INDIRECT(N141&amp;L143)&amp;","&amp;INDIRECT(N141&amp;L144)&amp;",1,-1,NONE,NONE,LNO MINISCAN "&amp;A138&amp;"KHZ STARTING ORDER "&amp;INDIRECT(M141&amp;L143)&amp;" &amp; "&amp;INDIRECT(M141&amp;L144)</f>
-        <v>3,1,272,273,1,-1,NONE,NONE,LNO MINISCAN 8KHZ STARTING ORDER 140 &amp; 146</v>
+    <row r="150" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B150" t="str">
+        <f ca="1">"3,1,"&amp;INDIRECT(D144&amp;B146)&amp;","&amp;INDIRECT(D144&amp;B147)&amp;",0,-1,NONE,NONE,SO MINISCAN "&amp;A141&amp;"KHZ STARTING ORDER "&amp;INDIRECT(C144&amp;B146)&amp;" &amp; "&amp;INDIRECT(C144&amp;B147)</f>
+        <v>3,1,220,221,0,-1,NONE,NONE,SO MINISCAN 8KHZ STARTING ORDER 110 &amp; 116</v>
+      </c>
+      <c r="L150" t="str">
+        <f ca="1">"3,1,"&amp;INDIRECT(N144&amp;L146)&amp;","&amp;INDIRECT(N144&amp;L147)&amp;",1,-1,NONE,NONE,LNO MINISCAN "&amp;A141&amp;"KHZ STARTING ORDER "&amp;INDIRECT(M144&amp;L146)&amp;" &amp; "&amp;INDIRECT(M144&amp;L147)</f>
+        <v>3,1,269,270,1,-1,NONE,NONE,LNO MINISCAN 8KHZ STARTING ORDER 122 &amp; 128</v>
       </c>
     </row>
   </sheetData>
@@ -7034,8 +7231,8 @@
     <mergeCell ref="F10:J10"/>
     <mergeCell ref="F17:J17"/>
     <mergeCell ref="P17:T17"/>
-    <mergeCell ref="F120:J120"/>
-    <mergeCell ref="P120:T120"/>
+    <mergeCell ref="F123:J123"/>
+    <mergeCell ref="P123:T123"/>
     <mergeCell ref="F86:J86"/>
     <mergeCell ref="P86:T86"/>
     <mergeCell ref="F52:J52"/>

</xml_diff>

<commit_message>
2026 patch done; MTP107 generated but dayside limb wrong
</commit_message>
<xml_diff>
--- a/observations/calibrations/solar_calibrations.xlsx
+++ b/observations/calibrations/solar_calibrations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iant\Documents\PROGRAMS\nomad_obs\observations\calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77CC3814-7648-4D5A-A5A1-1AFE76ECCB67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF300BE8-9F8C-4E0F-ABFF-15AB268DAB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -189,7 +189,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -390,6 +390,14 @@
       <u/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -911,7 +919,7 @@
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1029,6 +1037,24 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1041,35 +1067,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="18" builtinId="30" customBuiltin="1"/>
@@ -1597,13 +1596,13 @@
       <c r="E10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="91" t="s">
+      <c r="F10" s="99" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="92"/>
-      <c r="H10" s="92"/>
-      <c r="I10" s="92"/>
-      <c r="J10" s="92"/>
+      <c r="G10" s="100"/>
+      <c r="H10" s="100"/>
+      <c r="I10" s="100"/>
+      <c r="J10" s="100"/>
       <c r="K10" s="71"/>
       <c r="L10" s="71"/>
       <c r="M10" s="71"/>
@@ -1763,26 +1762,26 @@
       <c r="C17" s="13"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
-      <c r="F17" s="93" t="s">
+      <c r="F17" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="94"/>
-      <c r="H17" s="94"/>
-      <c r="I17" s="94"/>
-      <c r="J17" s="94"/>
+      <c r="G17" s="102"/>
+      <c r="H17" s="102"/>
+      <c r="I17" s="102"/>
+      <c r="J17" s="102"/>
       <c r="L17" s="9" t="s">
         <v>2</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="9"/>
       <c r="O17" s="9"/>
-      <c r="P17" s="93" t="s">
+      <c r="P17" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="Q17" s="94"/>
-      <c r="R17" s="94"/>
-      <c r="S17" s="94"/>
-      <c r="T17" s="94"/>
+      <c r="Q17" s="102"/>
+      <c r="R17" s="102"/>
+      <c r="S17" s="102"/>
+      <c r="T17" s="102"/>
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B18" s="39" t="s">
@@ -3355,26 +3354,26 @@
       <c r="C52" s="13"/>
       <c r="D52" s="9"/>
       <c r="E52" s="9"/>
-      <c r="F52" s="93" t="s">
+      <c r="F52" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="G52" s="94"/>
-      <c r="H52" s="94"/>
-      <c r="I52" s="94"/>
-      <c r="J52" s="94"/>
+      <c r="G52" s="102"/>
+      <c r="H52" s="102"/>
+      <c r="I52" s="102"/>
+      <c r="J52" s="102"/>
       <c r="L52" s="9" t="s">
         <v>2</v>
       </c>
       <c r="M52" s="13"/>
       <c r="N52" s="9"/>
       <c r="O52" s="9"/>
-      <c r="P52" s="93" t="s">
+      <c r="P52" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="Q52" s="94"/>
-      <c r="R52" s="94"/>
-      <c r="S52" s="94"/>
-      <c r="T52" s="94"/>
+      <c r="Q52" s="102"/>
+      <c r="R52" s="102"/>
+      <c r="S52" s="102"/>
+      <c r="T52" s="102"/>
     </row>
     <row r="53" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B53" s="9" t="s">
@@ -4640,26 +4639,26 @@
       <c r="C86" s="13"/>
       <c r="D86" s="9"/>
       <c r="E86" s="33"/>
-      <c r="F86" s="93" t="s">
+      <c r="F86" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="G86" s="94"/>
-      <c r="H86" s="94"/>
-      <c r="I86" s="94"/>
-      <c r="J86" s="94"/>
+      <c r="G86" s="102"/>
+      <c r="H86" s="102"/>
+      <c r="I86" s="102"/>
+      <c r="J86" s="102"/>
       <c r="L86" s="9" t="s">
         <v>2</v>
       </c>
       <c r="M86" s="13"/>
       <c r="N86" s="9"/>
       <c r="O86" s="33"/>
-      <c r="P86" s="93" t="s">
+      <c r="P86" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="Q86" s="94"/>
-      <c r="R86" s="94"/>
-      <c r="S86" s="94"/>
-      <c r="T86" s="94"/>
+      <c r="Q86" s="102"/>
+      <c r="R86" s="102"/>
+      <c r="S86" s="102"/>
+      <c r="T86" s="102"/>
     </row>
     <row r="87" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B87" s="9" t="s">
@@ -4727,7 +4726,7 @@
       <c r="C88" s="44">
         <v>386</v>
       </c>
-      <c r="D88" s="108">
+      <c r="D88" s="95">
         <v>370</v>
       </c>
       <c r="E88" s="26">
@@ -4770,20 +4769,18 @@
         <f>C88+2</f>
         <v>388</v>
       </c>
-      <c r="D89" s="97">
+      <c r="D89" s="90">
         <v>371</v>
       </c>
       <c r="E89" s="25">
         <v>190</v>
       </c>
-      <c r="F89" s="98">
+      <c r="F89" s="3">
         <v>9</v>
       </c>
-      <c r="G89" s="98">
+      <c r="G89" s="3">
         <v>80</v>
       </c>
-      <c r="H89" s="95"/>
-      <c r="I89" s="95"/>
       <c r="J89" s="4"/>
       <c r="L89" s="5">
         <f>L88+3</f>
@@ -4796,15 +4793,12 @@
       <c r="N89" s="59">
         <v>404</v>
       </c>
-      <c r="O89" s="95">
+      <c r="O89">
         <v>237</v>
       </c>
       <c r="P89" s="2">
         <v>9</v>
       </c>
-      <c r="Q89" s="95"/>
-      <c r="R89" s="95"/>
-      <c r="S89" s="95"/>
       <c r="T89" s="4"/>
     </row>
     <row r="90" spans="1:20" x14ac:dyDescent="0.3">
@@ -4819,22 +4813,22 @@
         <f t="shared" ref="C90:C115" si="6">C89+2</f>
         <v>390</v>
       </c>
-      <c r="D90" s="109">
+      <c r="D90" s="96">
         <v>372</v>
       </c>
-      <c r="E90" s="107">
+      <c r="E90" s="94">
         <v>191</v>
       </c>
-      <c r="F90" s="99">
+      <c r="F90" s="32">
         <v>7</v>
       </c>
-      <c r="G90" s="99">
+      <c r="G90" s="32">
         <v>57</v>
       </c>
-      <c r="H90" s="99">
+      <c r="H90" s="32">
         <v>80</v>
       </c>
-      <c r="I90" s="100"/>
+      <c r="I90" s="30"/>
       <c r="J90" s="31"/>
       <c r="K90" s="30"/>
       <c r="L90" s="29">
@@ -4848,15 +4842,15 @@
       <c r="N90" s="60">
         <v>405</v>
       </c>
-      <c r="O90" s="98">
+      <c r="O90" s="3">
         <v>238</v>
       </c>
       <c r="P90" s="29">
         <v>7</v>
       </c>
-      <c r="Q90" s="100"/>
-      <c r="R90" s="100"/>
-      <c r="S90" s="100"/>
+      <c r="Q90" s="30"/>
+      <c r="R90" s="30"/>
+      <c r="S90" s="30"/>
       <c r="T90" s="31"/>
     </row>
     <row r="91" spans="1:20" x14ac:dyDescent="0.3">
@@ -4871,22 +4865,22 @@
         <f t="shared" si="6"/>
         <v>392</v>
       </c>
-      <c r="D91" s="110">
+      <c r="D91" s="97">
         <v>373</v>
       </c>
       <c r="E91" s="74">
         <v>192</v>
       </c>
-      <c r="F91" s="102">
+      <c r="F91" s="79">
         <v>57</v>
       </c>
-      <c r="G91" s="102">
+      <c r="G91" s="79">
         <v>81</v>
       </c>
-      <c r="H91" s="102">
+      <c r="H91" s="79">
         <v>86</v>
       </c>
-      <c r="I91" s="101"/>
+      <c r="I91" s="73"/>
       <c r="J91" s="85"/>
       <c r="L91" s="35">
         <f t="shared" si="7"/>
@@ -4899,15 +4893,12 @@
       <c r="N91" s="75">
         <v>406</v>
       </c>
-      <c r="O91" s="101">
+      <c r="O91" s="73">
         <v>239</v>
       </c>
       <c r="P91" s="5">
         <v>60</v>
       </c>
-      <c r="Q91" s="95"/>
-      <c r="R91" s="95"/>
-      <c r="S91" s="95"/>
       <c r="T91" s="4"/>
     </row>
     <row r="92" spans="1:20" x14ac:dyDescent="0.3">
@@ -4922,18 +4913,15 @@
         <f t="shared" si="6"/>
         <v>394</v>
       </c>
-      <c r="D92" s="97">
+      <c r="D92" s="90">
         <v>374</v>
       </c>
       <c r="E92" s="25">
         <v>193</v>
       </c>
-      <c r="F92" s="98">
+      <c r="F92" s="3">
         <v>81</v>
       </c>
-      <c r="G92" s="95"/>
-      <c r="H92" s="95"/>
-      <c r="I92" s="95"/>
       <c r="J92" s="4"/>
       <c r="L92" s="5">
         <f t="shared" si="7"/>
@@ -4946,13 +4934,10 @@
       <c r="N92" s="59">
         <v>407</v>
       </c>
-      <c r="O92" s="95">
+      <c r="O92">
         <v>240</v>
       </c>
       <c r="P92" s="5"/>
-      <c r="Q92" s="95"/>
-      <c r="R92" s="95"/>
-      <c r="S92" s="95"/>
       <c r="T92" s="4"/>
     </row>
     <row r="93" spans="1:20" x14ac:dyDescent="0.3">
@@ -4967,18 +4952,15 @@
         <f t="shared" si="6"/>
         <v>396</v>
       </c>
-      <c r="D93" s="97">
+      <c r="D93" s="90">
         <v>375</v>
       </c>
       <c r="E93" s="25">
         <v>194</v>
       </c>
-      <c r="F93" s="98">
+      <c r="F93" s="3">
         <v>100</v>
       </c>
-      <c r="G93" s="95"/>
-      <c r="H93" s="95"/>
-      <c r="I93" s="95"/>
       <c r="J93" s="4"/>
       <c r="L93" s="5">
         <f t="shared" si="7"/>
@@ -4991,13 +4973,10 @@
       <c r="N93" s="59">
         <v>408</v>
       </c>
-      <c r="O93" s="95">
+      <c r="O93">
         <v>241</v>
       </c>
       <c r="P93" s="5"/>
-      <c r="Q93" s="95"/>
-      <c r="R93" s="95"/>
-      <c r="S93" s="95"/>
       <c r="T93" s="4"/>
     </row>
     <row r="94" spans="1:20" x14ac:dyDescent="0.3">
@@ -5012,20 +4991,18 @@
         <f t="shared" si="6"/>
         <v>398</v>
       </c>
-      <c r="D94" s="97">
+      <c r="D94" s="90">
         <v>376</v>
       </c>
       <c r="E94" s="25">
         <v>195</v>
       </c>
-      <c r="F94" s="98">
+      <c r="F94" s="3">
         <v>9</v>
       </c>
-      <c r="G94" s="98">
+      <c r="G94" s="3">
         <v>82</v>
       </c>
-      <c r="H94" s="95"/>
-      <c r="I94" s="95"/>
       <c r="J94" s="4"/>
       <c r="L94" s="5">
         <f t="shared" si="7"/>
@@ -5038,15 +5015,12 @@
       <c r="N94" s="59">
         <v>409</v>
       </c>
-      <c r="O94" s="95">
+      <c r="O94">
         <v>242</v>
       </c>
       <c r="P94" s="2">
         <v>9</v>
       </c>
-      <c r="Q94" s="95"/>
-      <c r="R94" s="95"/>
-      <c r="S94" s="95"/>
       <c r="T94" s="4"/>
     </row>
     <row r="95" spans="1:20" x14ac:dyDescent="0.3">
@@ -5061,22 +5035,22 @@
         <f t="shared" si="6"/>
         <v>400</v>
       </c>
-      <c r="D95" s="111">
+      <c r="D95" s="98">
         <v>377</v>
       </c>
       <c r="E95" s="77">
         <v>196</v>
       </c>
-      <c r="F95" s="103">
+      <c r="F95" s="82">
         <v>7</v>
       </c>
-      <c r="G95" s="103">
+      <c r="G95" s="82">
         <v>15</v>
       </c>
-      <c r="H95" s="103">
+      <c r="H95" s="82">
         <v>82</v>
       </c>
-      <c r="I95" s="104"/>
+      <c r="I95" s="91"/>
       <c r="J95" s="86"/>
       <c r="K95" s="30"/>
       <c r="L95" s="80">
@@ -5090,17 +5064,17 @@
       <c r="N95" s="78">
         <v>410</v>
       </c>
-      <c r="O95" s="102">
+      <c r="O95" s="79">
         <v>243</v>
       </c>
       <c r="P95" s="29">
         <v>7</v>
       </c>
-      <c r="Q95" s="99">
+      <c r="Q95" s="32">
         <v>15</v>
       </c>
-      <c r="R95" s="100"/>
-      <c r="S95" s="100"/>
+      <c r="R95" s="30"/>
+      <c r="S95" s="30"/>
       <c r="T95" s="31"/>
     </row>
     <row r="96" spans="1:20" x14ac:dyDescent="0.3">
@@ -5115,18 +5089,15 @@
         <f t="shared" si="6"/>
         <v>402</v>
       </c>
-      <c r="D96" s="97">
+      <c r="D96" s="90">
         <v>378</v>
       </c>
       <c r="E96" s="25">
         <v>197</v>
       </c>
-      <c r="F96" s="98">
+      <c r="F96" s="3">
         <v>82</v>
       </c>
-      <c r="G96" s="95"/>
-      <c r="H96" s="95"/>
-      <c r="I96" s="95"/>
       <c r="J96" s="4"/>
       <c r="L96" s="5">
         <f t="shared" si="7"/>
@@ -5139,15 +5110,12 @@
       <c r="N96" s="59">
         <v>411</v>
       </c>
-      <c r="O96" s="95">
+      <c r="O96">
         <v>244</v>
       </c>
       <c r="P96" s="2">
         <v>39</v>
       </c>
-      <c r="Q96" s="95"/>
-      <c r="R96" s="95"/>
-      <c r="S96" s="95"/>
       <c r="T96" s="4"/>
     </row>
     <row r="97" spans="1:20" x14ac:dyDescent="0.3">
@@ -5162,22 +5130,22 @@
         <f t="shared" si="6"/>
         <v>404</v>
       </c>
-      <c r="D97" s="111">
+      <c r="D97" s="98">
         <v>379</v>
       </c>
       <c r="E97" s="77">
         <v>198</v>
       </c>
-      <c r="F97" s="103">
+      <c r="F97" s="82">
         <v>8</v>
       </c>
-      <c r="G97" s="103">
+      <c r="G97" s="82">
         <v>21</v>
       </c>
-      <c r="H97" s="103">
+      <c r="H97" s="82">
         <v>82</v>
       </c>
-      <c r="I97" s="104"/>
+      <c r="I97" s="91"/>
       <c r="J97" s="86"/>
       <c r="K97" s="30"/>
       <c r="L97" s="80">
@@ -5191,15 +5159,15 @@
       <c r="N97" s="78">
         <v>412</v>
       </c>
-      <c r="O97" s="102">
+      <c r="O97" s="79">
         <v>245</v>
       </c>
       <c r="P97" s="29">
         <v>8</v>
       </c>
-      <c r="Q97" s="100"/>
-      <c r="R97" s="100"/>
-      <c r="S97" s="100"/>
+      <c r="Q97" s="30"/>
+      <c r="R97" s="30"/>
+      <c r="S97" s="30"/>
       <c r="T97" s="31"/>
     </row>
     <row r="98" spans="1:20" x14ac:dyDescent="0.3">
@@ -5214,20 +5182,20 @@
         <f t="shared" si="6"/>
         <v>406</v>
       </c>
-      <c r="D98" s="109">
+      <c r="D98" s="96">
         <v>380</v>
       </c>
-      <c r="E98" s="107">
+      <c r="E98" s="94">
         <v>199</v>
       </c>
-      <c r="F98" s="99">
+      <c r="F98" s="32">
         <v>23</v>
       </c>
-      <c r="G98" s="99">
+      <c r="G98" s="32">
         <v>86</v>
       </c>
-      <c r="H98" s="100"/>
-      <c r="I98" s="100"/>
+      <c r="H98" s="30"/>
+      <c r="I98" s="30"/>
       <c r="J98" s="31"/>
       <c r="L98" s="29">
         <f t="shared" si="7"/>
@@ -5240,15 +5208,15 @@
       <c r="N98" s="60">
         <v>413</v>
       </c>
-      <c r="O98" s="98">
+      <c r="O98" s="3">
         <v>246</v>
       </c>
       <c r="P98" s="28">
         <v>60</v>
       </c>
-      <c r="Q98" s="100"/>
-      <c r="R98" s="100"/>
-      <c r="S98" s="100"/>
+      <c r="Q98" s="30"/>
+      <c r="R98" s="30"/>
+      <c r="S98" s="30"/>
       <c r="T98" s="31"/>
     </row>
     <row r="99" spans="1:20" x14ac:dyDescent="0.3">
@@ -5263,18 +5231,15 @@
         <f t="shared" si="6"/>
         <v>408</v>
       </c>
-      <c r="D99" s="97">
+      <c r="D99" s="90">
         <v>381</v>
       </c>
       <c r="E99" s="25">
         <v>200</v>
       </c>
-      <c r="F99" s="106">
+      <c r="F99" s="93">
         <v>100</v>
       </c>
-      <c r="G99" s="95"/>
-      <c r="H99" s="95"/>
-      <c r="I99" s="95"/>
       <c r="J99" s="4"/>
       <c r="L99" s="5">
         <f t="shared" si="7"/>
@@ -5287,15 +5252,12 @@
       <c r="N99" s="59">
         <v>414</v>
       </c>
-      <c r="O99" s="95">
+      <c r="O99">
         <v>247</v>
       </c>
       <c r="P99" s="35">
         <v>60</v>
       </c>
-      <c r="Q99" s="95"/>
-      <c r="R99" s="95"/>
-      <c r="S99" s="95"/>
       <c r="T99" s="4"/>
     </row>
     <row r="100" spans="1:20" x14ac:dyDescent="0.3">
@@ -5310,18 +5272,15 @@
         <f t="shared" si="6"/>
         <v>410</v>
       </c>
-      <c r="D100" s="97">
+      <c r="D100" s="90">
         <v>382</v>
       </c>
       <c r="E100" s="25">
         <v>201</v>
       </c>
-      <c r="F100" s="98">
+      <c r="F100" s="3">
         <v>100</v>
       </c>
-      <c r="G100" s="95"/>
-      <c r="H100" s="95"/>
-      <c r="I100" s="95"/>
       <c r="J100" s="4"/>
       <c r="L100" s="5">
         <f t="shared" si="7"/>
@@ -5334,15 +5293,12 @@
       <c r="N100" s="59">
         <v>415</v>
       </c>
-      <c r="O100" s="95">
+      <c r="O100">
         <v>248</v>
       </c>
       <c r="P100" s="5">
         <v>60</v>
       </c>
-      <c r="Q100" s="95"/>
-      <c r="R100" s="95"/>
-      <c r="S100" s="95"/>
       <c r="T100" s="4"/>
     </row>
     <row r="101" spans="1:20" x14ac:dyDescent="0.3">
@@ -5357,18 +5313,15 @@
         <f t="shared" si="6"/>
         <v>412</v>
       </c>
-      <c r="D101" s="97">
+      <c r="D101" s="90">
         <v>383</v>
       </c>
       <c r="E101" s="25">
         <v>202</v>
       </c>
-      <c r="F101" s="98">
+      <c r="F101" s="3">
         <v>9</v>
       </c>
-      <c r="G101" s="95"/>
-      <c r="H101" s="95"/>
-      <c r="I101" s="95"/>
       <c r="J101" s="4"/>
       <c r="L101" s="5">
         <f t="shared" si="7"/>
@@ -5381,15 +5334,12 @@
       <c r="N101" s="59">
         <v>416</v>
       </c>
-      <c r="O101" s="95">
+      <c r="O101">
         <v>249</v>
       </c>
       <c r="P101" s="2">
         <v>9</v>
       </c>
-      <c r="Q101" s="95"/>
-      <c r="R101" s="95"/>
-      <c r="S101" s="95"/>
       <c r="T101" s="4"/>
     </row>
     <row r="102" spans="1:20" x14ac:dyDescent="0.3">
@@ -5404,20 +5354,20 @@
         <f t="shared" si="6"/>
         <v>414</v>
       </c>
-      <c r="D102" s="109">
+      <c r="D102" s="96">
         <v>384</v>
       </c>
-      <c r="E102" s="107">
+      <c r="E102" s="94">
         <v>203</v>
       </c>
-      <c r="F102" s="99">
+      <c r="F102" s="32">
         <v>8</v>
       </c>
-      <c r="G102" s="99">
+      <c r="G102" s="32">
         <v>21</v>
       </c>
-      <c r="H102" s="100"/>
-      <c r="I102" s="100"/>
+      <c r="H102" s="30"/>
+      <c r="I102" s="30"/>
       <c r="J102" s="31"/>
       <c r="K102" s="30"/>
       <c r="L102" s="29">
@@ -5431,17 +5381,17 @@
       <c r="N102" s="60">
         <v>417</v>
       </c>
-      <c r="O102" s="98">
+      <c r="O102" s="3">
         <v>250</v>
       </c>
       <c r="P102" s="29">
         <v>8</v>
       </c>
-      <c r="Q102" s="99">
+      <c r="Q102" s="32">
         <v>85</v>
       </c>
-      <c r="R102" s="100"/>
-      <c r="S102" s="100"/>
+      <c r="R102" s="30"/>
+      <c r="S102" s="30"/>
       <c r="T102" s="31"/>
     </row>
     <row r="103" spans="1:20" x14ac:dyDescent="0.3">
@@ -5456,20 +5406,20 @@
         <f t="shared" si="6"/>
         <v>416</v>
       </c>
-      <c r="D103" s="110">
+      <c r="D103" s="97">
         <v>385</v>
       </c>
       <c r="E103" s="74">
         <v>204</v>
       </c>
-      <c r="F103" s="102">
+      <c r="F103" s="79">
         <v>47</v>
       </c>
-      <c r="G103" s="102">
+      <c r="G103" s="79">
         <v>95</v>
       </c>
-      <c r="H103" s="101"/>
-      <c r="I103" s="101"/>
+      <c r="H103" s="73"/>
+      <c r="I103" s="73"/>
       <c r="J103" s="85"/>
       <c r="L103" s="35">
         <f t="shared" si="7"/>
@@ -5482,17 +5432,15 @@
       <c r="N103" s="75">
         <v>418</v>
       </c>
-      <c r="O103" s="101">
+      <c r="O103" s="73">
         <v>251</v>
       </c>
       <c r="P103" s="2">
         <v>55</v>
       </c>
-      <c r="Q103" s="102">
+      <c r="Q103" s="79">
         <v>85</v>
       </c>
-      <c r="R103" s="95"/>
-      <c r="S103" s="95"/>
       <c r="T103" s="4"/>
     </row>
     <row r="104" spans="1:20" x14ac:dyDescent="0.3">
@@ -5507,20 +5455,20 @@
         <f t="shared" si="6"/>
         <v>418</v>
       </c>
-      <c r="D104" s="110">
+      <c r="D104" s="97">
         <v>386</v>
       </c>
       <c r="E104" s="74">
         <v>205</v>
       </c>
-      <c r="F104" s="102">
+      <c r="F104" s="79">
         <v>7</v>
       </c>
-      <c r="G104" s="102">
+      <c r="G104" s="79">
         <v>47</v>
       </c>
-      <c r="H104" s="101"/>
-      <c r="I104" s="101"/>
+      <c r="H104" s="73"/>
+      <c r="I104" s="73"/>
       <c r="J104" s="85"/>
       <c r="L104" s="81">
         <f t="shared" si="7"/>
@@ -5533,15 +5481,12 @@
       <c r="N104" s="78">
         <v>419</v>
       </c>
-      <c r="O104" s="101">
+      <c r="O104" s="73">
         <v>252</v>
       </c>
       <c r="P104" s="2">
         <v>7</v>
       </c>
-      <c r="Q104" s="95"/>
-      <c r="R104" s="95"/>
-      <c r="S104" s="95"/>
       <c r="T104" s="4"/>
     </row>
     <row r="105" spans="1:20" x14ac:dyDescent="0.3">
@@ -5556,20 +5501,18 @@
         <f t="shared" si="6"/>
         <v>420</v>
       </c>
-      <c r="D105" s="97">
+      <c r="D105" s="90">
         <v>387</v>
       </c>
       <c r="E105" s="25">
         <v>206</v>
       </c>
-      <c r="F105" s="98">
+      <c r="F105" s="3">
         <v>8</v>
       </c>
-      <c r="G105" s="98">
+      <c r="G105" s="3">
         <v>57</v>
       </c>
-      <c r="H105" s="95"/>
-      <c r="I105" s="95"/>
       <c r="J105" s="4"/>
       <c r="L105" s="5">
         <f t="shared" si="7"/>
@@ -5582,15 +5525,12 @@
       <c r="N105" s="59">
         <v>420</v>
       </c>
-      <c r="O105" s="95">
+      <c r="O105">
         <v>253</v>
       </c>
       <c r="P105" s="2">
         <v>8</v>
       </c>
-      <c r="Q105" s="95"/>
-      <c r="R105" s="95"/>
-      <c r="S105" s="95"/>
       <c r="T105" s="4"/>
     </row>
     <row r="106" spans="1:20" x14ac:dyDescent="0.3">
@@ -5605,20 +5545,18 @@
         <f t="shared" si="6"/>
         <v>422</v>
       </c>
-      <c r="D106" s="97">
+      <c r="D106" s="90">
         <v>388</v>
       </c>
       <c r="E106" s="25">
         <v>207</v>
       </c>
-      <c r="F106" s="98">
+      <c r="F106" s="3">
         <v>27</v>
       </c>
-      <c r="G106" s="98">
+      <c r="G106" s="3">
         <v>57</v>
       </c>
-      <c r="H106" s="95"/>
-      <c r="I106" s="95"/>
       <c r="J106" s="4"/>
       <c r="L106" s="5">
         <f t="shared" si="7"/>
@@ -5631,15 +5569,12 @@
       <c r="N106" s="59">
         <v>421</v>
       </c>
-      <c r="O106" s="95">
+      <c r="O106">
         <v>254</v>
       </c>
       <c r="P106" s="2">
         <v>39</v>
       </c>
-      <c r="Q106" s="95"/>
-      <c r="R106" s="95"/>
-      <c r="S106" s="95"/>
       <c r="T106" s="4"/>
     </row>
     <row r="107" spans="1:20" x14ac:dyDescent="0.3">
@@ -5654,20 +5589,18 @@
         <f t="shared" si="6"/>
         <v>424</v>
       </c>
-      <c r="D107" s="97">
+      <c r="D107" s="90">
         <v>389</v>
       </c>
       <c r="E107" s="25">
         <v>208</v>
       </c>
-      <c r="F107" s="98">
+      <c r="F107" s="3">
         <v>27</v>
       </c>
-      <c r="G107" s="98">
+      <c r="G107" s="3">
         <v>88</v>
       </c>
-      <c r="H107" s="95"/>
-      <c r="I107" s="95"/>
       <c r="J107" s="4"/>
       <c r="L107" s="5">
         <f t="shared" si="7"/>
@@ -5680,15 +5613,12 @@
       <c r="N107" s="59">
         <v>422</v>
       </c>
-      <c r="O107" s="95">
+      <c r="O107">
         <v>255</v>
       </c>
       <c r="P107" s="2">
         <v>55</v>
       </c>
-      <c r="Q107" s="95"/>
-      <c r="R107" s="95"/>
-      <c r="S107" s="95"/>
       <c r="T107" s="4"/>
     </row>
     <row r="108" spans="1:20" x14ac:dyDescent="0.3">
@@ -5703,20 +5633,18 @@
         <f t="shared" si="6"/>
         <v>426</v>
       </c>
-      <c r="D108" s="97">
+      <c r="D108" s="90">
         <v>390</v>
       </c>
       <c r="E108" s="25">
         <v>209</v>
       </c>
-      <c r="F108" s="98">
+      <c r="F108" s="3">
         <v>27</v>
       </c>
-      <c r="G108" s="98">
+      <c r="G108" s="3">
         <v>88</v>
       </c>
-      <c r="H108" s="95"/>
-      <c r="I108" s="95"/>
       <c r="J108" s="4"/>
       <c r="L108" s="5">
         <f t="shared" si="7"/>
@@ -5729,15 +5657,12 @@
       <c r="N108" s="59">
         <v>423</v>
       </c>
-      <c r="O108" s="95">
+      <c r="O108">
         <v>256</v>
       </c>
       <c r="P108" s="2">
         <v>55</v>
       </c>
-      <c r="Q108" s="95"/>
-      <c r="R108" s="95"/>
-      <c r="S108" s="95"/>
       <c r="T108" s="4"/>
     </row>
     <row r="109" spans="1:20" x14ac:dyDescent="0.3">
@@ -5752,20 +5677,18 @@
         <f t="shared" si="6"/>
         <v>428</v>
       </c>
-      <c r="D109" s="97">
+      <c r="D109" s="90">
         <v>391</v>
       </c>
       <c r="E109" s="25">
         <v>210</v>
       </c>
-      <c r="F109" s="98">
+      <c r="F109" s="3">
         <v>27</v>
       </c>
-      <c r="G109" s="98">
+      <c r="G109" s="3">
         <v>105</v>
       </c>
-      <c r="H109" s="95"/>
-      <c r="I109" s="95"/>
       <c r="J109" s="4"/>
       <c r="L109" s="5">
         <f t="shared" si="7"/>
@@ -5778,15 +5701,12 @@
       <c r="N109" s="59">
         <v>424</v>
       </c>
-      <c r="O109" s="95">
+      <c r="O109">
         <v>257</v>
       </c>
       <c r="P109" s="2">
         <v>55</v>
       </c>
-      <c r="Q109" s="95"/>
-      <c r="R109" s="95"/>
-      <c r="S109" s="95"/>
       <c r="T109" s="4"/>
     </row>
     <row r="110" spans="1:20" x14ac:dyDescent="0.3">
@@ -5801,20 +5721,18 @@
         <f t="shared" si="6"/>
         <v>430</v>
       </c>
-      <c r="D110" s="97">
+      <c r="D110" s="90">
         <v>392</v>
       </c>
       <c r="E110" s="25">
         <v>211</v>
       </c>
-      <c r="F110" s="98">
+      <c r="F110" s="3">
         <v>38</v>
       </c>
-      <c r="G110" s="98">
+      <c r="G110" s="3">
         <v>95</v>
       </c>
-      <c r="H110" s="95"/>
-      <c r="I110" s="95"/>
       <c r="J110" s="4"/>
       <c r="L110" s="5">
         <f t="shared" si="7"/>
@@ -5827,15 +5745,12 @@
       <c r="N110" s="59">
         <v>425</v>
       </c>
-      <c r="O110" s="95">
+      <c r="O110">
         <v>258</v>
       </c>
       <c r="P110" s="2">
         <v>38</v>
       </c>
-      <c r="Q110" s="95"/>
-      <c r="R110" s="95"/>
-      <c r="S110" s="95"/>
       <c r="T110" s="4"/>
     </row>
     <row r="111" spans="1:20" x14ac:dyDescent="0.3">
@@ -5850,22 +5765,22 @@
         <f t="shared" si="6"/>
         <v>432</v>
       </c>
-      <c r="D111" s="110">
+      <c r="D111" s="97">
         <v>393</v>
       </c>
       <c r="E111" s="74">
         <v>212</v>
       </c>
-      <c r="F111" s="102">
+      <c r="F111" s="79">
         <v>38</v>
       </c>
-      <c r="G111" s="102">
+      <c r="G111" s="79">
         <v>47</v>
       </c>
-      <c r="H111" s="102">
+      <c r="H111" s="79">
         <v>62</v>
       </c>
-      <c r="I111" s="102">
+      <c r="I111" s="79">
         <v>78</v>
       </c>
       <c r="J111" s="85"/>
@@ -5880,17 +5795,15 @@
       <c r="N111" s="75">
         <v>426</v>
       </c>
-      <c r="O111" s="101">
+      <c r="O111" s="73">
         <v>259</v>
       </c>
       <c r="P111" s="2">
         <v>38</v>
       </c>
-      <c r="Q111" s="102">
+      <c r="Q111" s="79">
         <v>84</v>
       </c>
-      <c r="R111" s="95"/>
-      <c r="S111" s="95"/>
       <c r="T111" s="4"/>
     </row>
     <row r="112" spans="1:20" x14ac:dyDescent="0.3">
@@ -5905,22 +5818,22 @@
         <f t="shared" si="6"/>
         <v>434</v>
       </c>
-      <c r="D112" s="97">
+      <c r="D112" s="90">
         <v>394</v>
       </c>
       <c r="E112" s="25">
         <v>213</v>
       </c>
-      <c r="F112" s="98">
+      <c r="F112" s="3">
         <v>9</v>
       </c>
-      <c r="G112" s="98">
+      <c r="G112" s="3">
         <v>47</v>
       </c>
-      <c r="H112" s="98">
+      <c r="H112" s="3">
         <v>62</v>
       </c>
-      <c r="I112" s="98">
+      <c r="I112" s="3">
         <v>78</v>
       </c>
       <c r="J112" s="4"/>
@@ -5935,17 +5848,15 @@
       <c r="N112" s="59">
         <v>427</v>
       </c>
-      <c r="O112" s="95">
+      <c r="O112">
         <v>260</v>
       </c>
       <c r="P112" s="2">
         <v>9</v>
       </c>
-      <c r="Q112" s="98">
+      <c r="Q112" s="3">
         <v>84</v>
       </c>
-      <c r="R112" s="95"/>
-      <c r="S112" s="95"/>
       <c r="T112" s="4"/>
     </row>
     <row r="113" spans="1:20" x14ac:dyDescent="0.3">
@@ -5960,22 +5871,22 @@
         <f t="shared" si="6"/>
         <v>436</v>
       </c>
-      <c r="D113" s="111">
+      <c r="D113" s="98">
         <v>395</v>
       </c>
       <c r="E113" s="77">
         <v>214</v>
       </c>
-      <c r="F113" s="103">
+      <c r="F113" s="82">
         <v>7</v>
       </c>
-      <c r="G113" s="103">
+      <c r="G113" s="82">
         <v>13</v>
       </c>
-      <c r="H113" s="103">
+      <c r="H113" s="82">
         <v>78</v>
       </c>
-      <c r="I113" s="104"/>
+      <c r="I113" s="103"/>
       <c r="J113" s="86"/>
       <c r="K113" s="30"/>
       <c r="L113" s="80">
@@ -5989,17 +5900,17 @@
       <c r="N113" s="78">
         <v>428</v>
       </c>
-      <c r="O113" s="102">
+      <c r="O113" s="79">
         <v>261</v>
       </c>
       <c r="P113" s="29">
         <v>7</v>
       </c>
-      <c r="Q113" s="99">
+      <c r="Q113" s="32">
         <v>13</v>
       </c>
-      <c r="R113" s="100"/>
-      <c r="S113" s="100"/>
+      <c r="R113" s="30"/>
+      <c r="S113" s="30"/>
       <c r="T113" s="31"/>
     </row>
     <row r="114" spans="1:20" x14ac:dyDescent="0.3">
@@ -6014,22 +5925,24 @@
         <f t="shared" si="6"/>
         <v>438</v>
       </c>
-      <c r="D114" s="110">
+      <c r="D114" s="97">
         <v>396</v>
       </c>
       <c r="E114" s="74">
         <v>215</v>
       </c>
-      <c r="F114" s="102">
+      <c r="F114" s="79">
         <v>8</v>
       </c>
-      <c r="G114" s="102">
+      <c r="G114" s="79">
         <v>78</v>
       </c>
-      <c r="H114" s="102">
+      <c r="H114" s="79">
         <v>105</v>
       </c>
-      <c r="I114" s="101"/>
+      <c r="I114" s="104">
+        <v>107</v>
+      </c>
       <c r="J114" s="85"/>
       <c r="L114" s="35">
         <f t="shared" si="7"/>
@@ -6042,15 +5955,13 @@
       <c r="N114" s="75">
         <v>429</v>
       </c>
-      <c r="O114" s="101">
+      <c r="O114" s="73">
         <v>262</v>
       </c>
       <c r="P114" s="2">
         <v>8</v>
       </c>
-      <c r="Q114" s="101"/>
-      <c r="R114" s="95"/>
-      <c r="S114" s="95"/>
+      <c r="Q114" s="73"/>
       <c r="T114" s="4"/>
     </row>
     <row r="115" spans="1:20" x14ac:dyDescent="0.3">
@@ -6065,22 +5976,22 @@
         <f t="shared" si="6"/>
         <v>440</v>
       </c>
-      <c r="D115" s="97">
+      <c r="D115" s="90">
         <v>397</v>
       </c>
       <c r="E115" s="25">
         <v>216</v>
       </c>
-      <c r="F115" s="98">
+      <c r="F115" s="3">
         <v>96</v>
       </c>
-      <c r="G115" s="98">
+      <c r="G115" s="3">
         <v>96</v>
       </c>
-      <c r="H115" s="98">
+      <c r="H115" s="3">
         <v>97</v>
       </c>
-      <c r="I115" s="98"/>
+      <c r="I115" s="3"/>
       <c r="J115" s="4"/>
       <c r="L115" s="5">
         <f t="shared" si="7"/>
@@ -6093,13 +6004,10 @@
       <c r="N115" s="59">
         <v>430</v>
       </c>
-      <c r="O115" s="95">
+      <c r="O115">
         <v>263</v>
       </c>
       <c r="P115" s="5"/>
-      <c r="Q115" s="95"/>
-      <c r="R115" s="95"/>
-      <c r="S115" s="95"/>
       <c r="T115" s="4"/>
     </row>
     <row r="116" spans="1:20" x14ac:dyDescent="0.3">
@@ -6114,22 +6022,21 @@
         <f>C115+2</f>
         <v>442</v>
       </c>
-      <c r="D116" s="97">
+      <c r="D116" s="90">
         <v>398</v>
       </c>
       <c r="E116" s="25">
         <v>217</v>
       </c>
-      <c r="F116" s="98">
+      <c r="F116" s="3">
         <v>96</v>
       </c>
-      <c r="G116" s="98">
+      <c r="G116" s="3">
         <v>96</v>
       </c>
-      <c r="H116" s="98">
+      <c r="H116" s="3">
         <v>97</v>
       </c>
-      <c r="I116" s="95"/>
       <c r="J116" s="4"/>
       <c r="L116" s="6">
         <f>L115+3</f>
@@ -6160,26 +6067,16 @@
         <v>206</v>
       </c>
       <c r="C117" s="42"/>
-      <c r="D117" s="97"/>
+      <c r="D117" s="90"/>
       <c r="E117" s="25">
         <v>218</v>
       </c>
-      <c r="F117" s="98">
+      <c r="F117" s="3">
         <v>106</v>
       </c>
-      <c r="G117" s="95"/>
-      <c r="H117" s="95"/>
-      <c r="I117" s="95"/>
       <c r="J117" s="4"/>
-      <c r="L117" s="95"/>
-      <c r="M117" s="96"/>
-      <c r="N117" s="97"/>
-      <c r="O117" s="95"/>
-      <c r="P117" s="95"/>
-      <c r="Q117" s="95"/>
-      <c r="R117" s="95"/>
-      <c r="S117" s="95"/>
-      <c r="T117" s="95"/>
+      <c r="M117" s="89"/>
+      <c r="N117" s="90"/>
     </row>
     <row r="118" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A118">
@@ -6190,26 +6087,21 @@
         <v>209</v>
       </c>
       <c r="C118" s="43"/>
-      <c r="D118" s="105"/>
+      <c r="D118" s="92"/>
       <c r="E118" s="34">
         <v>219</v>
       </c>
       <c r="F118" s="18">
         <v>106</v>
       </c>
-      <c r="G118" s="7"/>
+      <c r="G118" s="7">
+        <v>107</v>
+      </c>
       <c r="H118" s="7"/>
       <c r="I118" s="7"/>
       <c r="J118" s="8"/>
-      <c r="L118" s="95"/>
-      <c r="M118" s="96"/>
-      <c r="N118" s="97"/>
-      <c r="O118" s="95"/>
-      <c r="P118" s="95"/>
-      <c r="Q118" s="95"/>
-      <c r="R118" s="95"/>
-      <c r="S118" s="95"/>
-      <c r="T118" s="95"/>
+      <c r="M118" s="89"/>
+      <c r="N118" s="90"/>
     </row>
     <row r="119" spans="1:20" x14ac:dyDescent="0.3">
       <c r="C119" s="89"/>
@@ -6243,26 +6135,26 @@
       </c>
       <c r="C123" s="40"/>
       <c r="D123" s="9"/>
-      <c r="F123" s="93" t="s">
+      <c r="F123" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="G123" s="94"/>
-      <c r="H123" s="94"/>
-      <c r="I123" s="94"/>
-      <c r="J123" s="94"/>
+      <c r="G123" s="102"/>
+      <c r="H123" s="102"/>
+      <c r="I123" s="102"/>
+      <c r="J123" s="102"/>
       <c r="L123" s="9" t="s">
         <v>2</v>
       </c>
       <c r="M123" s="40"/>
       <c r="N123" s="9"/>
       <c r="O123" s="33"/>
-      <c r="P123" s="93" t="s">
+      <c r="P123" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="Q123" s="94"/>
-      <c r="R123" s="94"/>
-      <c r="S123" s="94"/>
-      <c r="T123" s="94"/>
+      <c r="Q123" s="102"/>
+      <c r="R123" s="102"/>
+      <c r="S123" s="102"/>
+      <c r="T123" s="102"/>
     </row>
     <row r="124" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B124" s="9" t="s">

</xml_diff>

<commit_message>
MTP107 done; new COP tables added to webdav; LTP019 filled in
</commit_message>
<xml_diff>
--- a/observations/calibrations/solar_calibrations.xlsx
+++ b/observations/calibrations/solar_calibrations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iant\Documents\PROGRAMS\nomad_obs\observations\calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF300BE8-9F8C-4E0F-ABFF-15AB268DAB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F92D13-75E3-4898-8647-9031C2CBA073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1635" yWindow="1425" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -919,7 +919,7 @@
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1055,6 +1055,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1067,8 +1068,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="18" builtinId="30" customBuiltin="1"/>
@@ -1391,23 +1390,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AE150"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" customWidth="1"/>
-    <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.109375" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" customWidth="1"/>
+    <col min="13" max="13" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="21" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.33203125" customWidth="1"/>
-    <col min="23" max="23" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.28515625" customWidth="1"/>
+    <col min="23" max="23" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:31" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1415,12 +1414,12 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="2:31" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
       <c r="W2" s="14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="2:31" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B3" s="14" t="s">
         <v>3</v>
       </c>
@@ -1433,7 +1432,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C4" s="13" t="s">
         <v>12</v>
       </c>
@@ -1472,7 +1471,7 @@
       <c r="AD4" s="71"/>
       <c r="AE4" s="65"/>
     </row>
-    <row r="5" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C5" s="19" t="s">
         <v>1</v>
       </c>
@@ -1514,7 +1513,7 @@
       </c>
       <c r="AE5" s="4"/>
     </row>
-    <row r="6" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C6" s="20" t="s">
         <v>2</v>
       </c>
@@ -1579,14 +1578,14 @@
       <c r="AD6" s="7"/>
       <c r="AE6" s="8"/>
     </row>
-    <row r="9" spans="2:31" ht="18" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="14" t="s">
         <v>24</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C10" s="13" t="s">
         <v>12</v>
       </c>
@@ -1596,13 +1595,13 @@
       <c r="E10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="99" t="s">
+      <c r="F10" s="100" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="100"/>
-      <c r="H10" s="100"/>
-      <c r="I10" s="100"/>
-      <c r="J10" s="100"/>
+      <c r="G10" s="101"/>
+      <c r="H10" s="101"/>
+      <c r="I10" s="101"/>
+      <c r="J10" s="101"/>
       <c r="K10" s="71"/>
       <c r="L10" s="71"/>
       <c r="M10" s="71"/>
@@ -1627,7 +1626,7 @@
       <c r="AD10" s="71"/>
       <c r="AE10" s="65"/>
     </row>
-    <row r="11" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C11" s="19" t="s">
         <v>34</v>
       </c>
@@ -1686,7 +1685,7 @@
       <c r="AD11" s="16"/>
       <c r="AE11" s="17"/>
     </row>
-    <row r="12" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C12" s="20" t="s">
         <v>36</v>
       </c>
@@ -1731,12 +1730,12 @@
       <c r="AD12" s="7"/>
       <c r="AE12" s="8"/>
     </row>
-    <row r="13" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="2:31" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B15" s="14" t="s">
         <v>0</v>
       </c>
@@ -1750,40 +1749,40 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:31" x14ac:dyDescent="0.25">
       <c r="AC16" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
-      <c r="F17" s="101" t="s">
+      <c r="F17" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="102"/>
-      <c r="H17" s="102"/>
-      <c r="I17" s="102"/>
-      <c r="J17" s="102"/>
+      <c r="G17" s="103"/>
+      <c r="H17" s="103"/>
+      <c r="I17" s="103"/>
+      <c r="J17" s="103"/>
       <c r="L17" s="9" t="s">
         <v>2</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="9"/>
       <c r="O17" s="9"/>
-      <c r="P17" s="101" t="s">
+      <c r="P17" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="Q17" s="102"/>
-      <c r="R17" s="102"/>
-      <c r="S17" s="102"/>
-      <c r="T17" s="102"/>
-    </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="Q17" s="103"/>
+      <c r="R17" s="103"/>
+      <c r="S17" s="103"/>
+      <c r="T17" s="103"/>
+    </row>
+    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B18" s="39" t="s">
         <v>10</v>
       </c>
@@ -1858,7 +1857,7 @@
       </c>
       <c r="AE18" s="9"/>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1</v>
       </c>
@@ -1913,7 +1912,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1</v>
       </c>
@@ -1962,7 +1961,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1</v>
       </c>
@@ -2009,7 +2008,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1</v>
       </c>
@@ -2073,7 +2072,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1</v>
       </c>
@@ -2122,7 +2121,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1</v>
       </c>
@@ -2171,7 +2170,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1</v>
       </c>
@@ -2231,7 +2230,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1</v>
       </c>
@@ -2280,7 +2279,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1</v>
       </c>
@@ -2332,7 +2331,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1</v>
       </c>
@@ -2377,7 +2376,7 @@
       </c>
       <c r="Z28" s="55"/>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1</v>
       </c>
@@ -2420,7 +2419,7 @@
       <c r="Y29" s="48"/>
       <c r="Z29" s="49"/>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1</v>
       </c>
@@ -2469,7 +2468,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>1</v>
       </c>
@@ -2514,7 +2513,7 @@
       <c r="Y31" s="48"/>
       <c r="Z31" s="49"/>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>1</v>
       </c>
@@ -2566,7 +2565,7 @@
       <c r="Y32" s="48"/>
       <c r="Z32" s="49"/>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>1</v>
       </c>
@@ -2611,7 +2610,7 @@
       <c r="Y33" s="48"/>
       <c r="Z33" s="49"/>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>1</v>
       </c>
@@ -2663,7 +2662,7 @@
       <c r="Y34" s="48"/>
       <c r="Z34" s="49"/>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>1</v>
       </c>
@@ -2709,7 +2708,7 @@
       <c r="Y35" s="48"/>
       <c r="Z35" s="49"/>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>1</v>
       </c>
@@ -2754,7 +2753,7 @@
       <c r="Y36" s="48"/>
       <c r="Z36" s="49"/>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>1</v>
       </c>
@@ -2797,7 +2796,7 @@
       <c r="Y37" s="48"/>
       <c r="Z37" s="49"/>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>1</v>
       </c>
@@ -2840,7 +2839,7 @@
       <c r="Y38" s="48"/>
       <c r="Z38" s="49"/>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>1</v>
       </c>
@@ -2886,7 +2885,7 @@
       <c r="Y39" s="48"/>
       <c r="Z39" s="49"/>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>1</v>
       </c>
@@ -2929,7 +2928,7 @@
       <c r="Y40" s="48"/>
       <c r="Z40" s="49"/>
     </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>1</v>
       </c>
@@ -2979,7 +2978,7 @@
       <c r="Y41" s="48"/>
       <c r="Z41" s="49"/>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>1</v>
       </c>
@@ -3030,7 +3029,7 @@
       <c r="Y42" s="48"/>
       <c r="Z42" s="49"/>
     </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>1</v>
       </c>
@@ -3085,7 +3084,7 @@
       <c r="Y43" s="48"/>
       <c r="Z43" s="49"/>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>1</v>
       </c>
@@ -3132,7 +3131,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>1</v>
       </c>
@@ -3178,7 +3177,7 @@
       <c r="Y45" s="5"/>
       <c r="Z45" s="4"/>
     </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>1</v>
       </c>
@@ -3219,7 +3218,7 @@
       <c r="Y46" s="5"/>
       <c r="Z46" s="4"/>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>1</v>
       </c>
@@ -3263,7 +3262,7 @@
       <c r="Y47" s="5"/>
       <c r="Z47" s="4"/>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>1</v>
       </c>
@@ -3314,7 +3313,7 @@
       <c r="Y48" s="5"/>
       <c r="Z48" s="4"/>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
       <c r="W49" s="5">
         <v>4526.9799999999996</v>
       </c>
@@ -3324,7 +3323,7 @@
       <c r="Y49" s="6"/>
       <c r="Z49" s="8"/>
     </row>
-    <row r="50" spans="1:26" ht="18" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:26" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B50" s="14" t="s">
         <v>0</v>
       </c>
@@ -3336,7 +3335,7 @@
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
     </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
       <c r="D51" s="1"/>
@@ -3347,35 +3346,35 @@
         <v>19</v>
       </c>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B52" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C52" s="13"/>
       <c r="D52" s="9"/>
       <c r="E52" s="9"/>
-      <c r="F52" s="101" t="s">
+      <c r="F52" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="G52" s="102"/>
-      <c r="H52" s="102"/>
-      <c r="I52" s="102"/>
-      <c r="J52" s="102"/>
+      <c r="G52" s="103"/>
+      <c r="H52" s="103"/>
+      <c r="I52" s="103"/>
+      <c r="J52" s="103"/>
       <c r="L52" s="9" t="s">
         <v>2</v>
       </c>
       <c r="M52" s="13"/>
       <c r="N52" s="9"/>
       <c r="O52" s="9"/>
-      <c r="P52" s="101" t="s">
+      <c r="P52" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="Q52" s="102"/>
-      <c r="R52" s="102"/>
-      <c r="S52" s="102"/>
-      <c r="T52" s="102"/>
-    </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="Q52" s="103"/>
+      <c r="R52" s="103"/>
+      <c r="S52" s="103"/>
+      <c r="T52" s="103"/>
+    </row>
+    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B53" s="9" t="s">
         <v>10</v>
       </c>
@@ -3431,7 +3430,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2</v>
       </c>
@@ -3468,7 +3467,7 @@
       </c>
       <c r="T54" s="4"/>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2</v>
       </c>
@@ -3505,7 +3504,7 @@
       <c r="P55" s="5"/>
       <c r="T55" s="4"/>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2</v>
       </c>
@@ -3557,7 +3556,7 @@
       <c r="S56" s="30"/>
       <c r="T56" s="31"/>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>2</v>
       </c>
@@ -3594,7 +3593,7 @@
       <c r="P57" s="5"/>
       <c r="T57" s="4"/>
     </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>2</v>
       </c>
@@ -3631,7 +3630,7 @@
       <c r="P58" s="5"/>
       <c r="T58" s="4"/>
     </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>2</v>
       </c>
@@ -3672,7 +3671,7 @@
       </c>
       <c r="T59" s="4"/>
     </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>2</v>
       </c>
@@ -3709,7 +3708,7 @@
       <c r="P60" s="5"/>
       <c r="T60" s="4"/>
     </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>2</v>
       </c>
@@ -3761,7 +3760,7 @@
       <c r="S61" s="30"/>
       <c r="T61" s="31"/>
     </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>2</v>
       </c>
@@ -3798,7 +3797,7 @@
       <c r="P62" s="5"/>
       <c r="T62" s="4"/>
     </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>2</v>
       </c>
@@ -3850,7 +3849,7 @@
       <c r="S63" s="30"/>
       <c r="T63" s="31"/>
     </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>2</v>
       </c>
@@ -3887,7 +3886,7 @@
       <c r="P64" s="5"/>
       <c r="T64" s="4"/>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>2</v>
       </c>
@@ -3924,7 +3923,7 @@
       <c r="P65" s="35"/>
       <c r="T65" s="4"/>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>2</v>
       </c>
@@ -3961,7 +3960,7 @@
       <c r="P66" s="5"/>
       <c r="T66" s="4"/>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>2</v>
       </c>
@@ -3998,7 +3997,7 @@
       <c r="P67" s="5"/>
       <c r="T67" s="4"/>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>2</v>
       </c>
@@ -4050,7 +4049,7 @@
       <c r="S68" s="30"/>
       <c r="T68" s="31"/>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>2</v>
       </c>
@@ -4097,7 +4096,7 @@
       </c>
       <c r="T69" s="4"/>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>2</v>
       </c>
@@ -4138,7 +4137,7 @@
       </c>
       <c r="T70" s="4"/>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>2</v>
       </c>
@@ -4175,7 +4174,7 @@
       <c r="P71" s="5"/>
       <c r="T71" s="4"/>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>2</v>
       </c>
@@ -4212,7 +4211,7 @@
       <c r="P72" s="5"/>
       <c r="T72" s="4"/>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>2</v>
       </c>
@@ -4249,7 +4248,7 @@
       <c r="P73" s="5"/>
       <c r="T73" s="4"/>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>2</v>
       </c>
@@ -4286,7 +4285,7 @@
       <c r="P74" s="5"/>
       <c r="T74" s="4"/>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>2</v>
       </c>
@@ -4323,7 +4322,7 @@
       <c r="P75" s="5"/>
       <c r="T75" s="4"/>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>2</v>
       </c>
@@ -4364,7 +4363,7 @@
       </c>
       <c r="T76" s="4"/>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>2</v>
       </c>
@@ -4408,7 +4407,7 @@
       </c>
       <c r="T77" s="4"/>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>2</v>
       </c>
@@ -4445,7 +4444,7 @@
       <c r="P78" s="5"/>
       <c r="T78" s="4"/>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>2</v>
       </c>
@@ -4493,7 +4492,7 @@
       <c r="S79" s="30"/>
       <c r="T79" s="31"/>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>2</v>
       </c>
@@ -4530,7 +4529,7 @@
       <c r="P80" s="5"/>
       <c r="T80" s="4"/>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>2</v>
       </c>
@@ -4567,7 +4566,7 @@
       <c r="P81" s="5"/>
       <c r="T81" s="4"/>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>2</v>
       </c>
@@ -4610,7 +4609,7 @@
       <c r="S82" s="7"/>
       <c r="T82" s="8"/>
     </row>
-    <row r="84" spans="1:20" ht="18" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B84" s="14" t="s">
         <v>0</v>
       </c>
@@ -4624,7 +4623,7 @@
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
       <c r="D85" s="1"/>
@@ -4632,35 +4631,35 @@
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B86" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C86" s="13"/>
       <c r="D86" s="9"/>
       <c r="E86" s="33"/>
-      <c r="F86" s="101" t="s">
+      <c r="F86" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="G86" s="102"/>
-      <c r="H86" s="102"/>
-      <c r="I86" s="102"/>
-      <c r="J86" s="102"/>
+      <c r="G86" s="103"/>
+      <c r="H86" s="103"/>
+      <c r="I86" s="103"/>
+      <c r="J86" s="103"/>
       <c r="L86" s="9" t="s">
         <v>2</v>
       </c>
       <c r="M86" s="13"/>
       <c r="N86" s="9"/>
       <c r="O86" s="33"/>
-      <c r="P86" s="101" t="s">
+      <c r="P86" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="Q86" s="102"/>
-      <c r="R86" s="102"/>
-      <c r="S86" s="102"/>
-      <c r="T86" s="102"/>
-    </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="Q86" s="103"/>
+      <c r="R86" s="103"/>
+      <c r="S86" s="103"/>
+      <c r="T86" s="103"/>
+    </row>
+    <row r="87" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B87" s="9" t="s">
         <v>10</v>
       </c>
@@ -4716,7 +4715,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>4</v>
       </c>
@@ -4757,7 +4756,7 @@
       <c r="S88" s="16"/>
       <c r="T88" s="17"/>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>4</v>
       </c>
@@ -4801,7 +4800,7 @@
       </c>
       <c r="T89" s="4"/>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>4</v>
       </c>
@@ -4853,7 +4852,7 @@
       <c r="S90" s="30"/>
       <c r="T90" s="31"/>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>4</v>
       </c>
@@ -4901,7 +4900,7 @@
       </c>
       <c r="T91" s="4"/>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>4</v>
       </c>
@@ -4940,7 +4939,7 @@
       <c r="P92" s="5"/>
       <c r="T92" s="4"/>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>4</v>
       </c>
@@ -4979,7 +4978,7 @@
       <c r="P93" s="5"/>
       <c r="T93" s="4"/>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>4</v>
       </c>
@@ -5023,7 +5022,7 @@
       </c>
       <c r="T94" s="4"/>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>4</v>
       </c>
@@ -5077,7 +5076,7 @@
       <c r="S95" s="30"/>
       <c r="T95" s="31"/>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>4</v>
       </c>
@@ -5118,7 +5117,7 @@
       </c>
       <c r="T96" s="4"/>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>4</v>
       </c>
@@ -5170,7 +5169,7 @@
       <c r="S97" s="30"/>
       <c r="T97" s="31"/>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>4</v>
       </c>
@@ -5219,7 +5218,7 @@
       <c r="S98" s="30"/>
       <c r="T98" s="31"/>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>4</v>
       </c>
@@ -5260,7 +5259,7 @@
       </c>
       <c r="T99" s="4"/>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>4</v>
       </c>
@@ -5301,7 +5300,7 @@
       </c>
       <c r="T100" s="4"/>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>4</v>
       </c>
@@ -5342,7 +5341,7 @@
       </c>
       <c r="T101" s="4"/>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>4</v>
       </c>
@@ -5394,7 +5393,7 @@
       <c r="S102" s="30"/>
       <c r="T102" s="31"/>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>4</v>
       </c>
@@ -5443,7 +5442,7 @@
       </c>
       <c r="T103" s="4"/>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>4</v>
       </c>
@@ -5489,7 +5488,7 @@
       </c>
       <c r="T104" s="4"/>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>4</v>
       </c>
@@ -5533,7 +5532,7 @@
       </c>
       <c r="T105" s="4"/>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>4</v>
       </c>
@@ -5577,7 +5576,7 @@
       </c>
       <c r="T106" s="4"/>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>4</v>
       </c>
@@ -5621,7 +5620,7 @@
       </c>
       <c r="T107" s="4"/>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>4</v>
       </c>
@@ -5665,7 +5664,7 @@
       </c>
       <c r="T108" s="4"/>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>4</v>
       </c>
@@ -5709,7 +5708,7 @@
       </c>
       <c r="T109" s="4"/>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>4</v>
       </c>
@@ -5753,7 +5752,7 @@
       </c>
       <c r="T110" s="4"/>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>4</v>
       </c>
@@ -5806,7 +5805,7 @@
       </c>
       <c r="T111" s="4"/>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>4</v>
       </c>
@@ -5859,7 +5858,7 @@
       </c>
       <c r="T112" s="4"/>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>4</v>
       </c>
@@ -5886,7 +5885,7 @@
       <c r="H113" s="82">
         <v>78</v>
       </c>
-      <c r="I113" s="103"/>
+      <c r="I113" s="99"/>
       <c r="J113" s="86"/>
       <c r="K113" s="30"/>
       <c r="L113" s="80">
@@ -5913,7 +5912,7 @@
       <c r="S113" s="30"/>
       <c r="T113" s="31"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>4</v>
       </c>
@@ -5940,7 +5939,7 @@
       <c r="H114" s="79">
         <v>105</v>
       </c>
-      <c r="I114" s="104">
+      <c r="I114" s="93">
         <v>107</v>
       </c>
       <c r="J114" s="85"/>
@@ -5964,7 +5963,7 @@
       <c r="Q114" s="73"/>
       <c r="T114" s="4"/>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>4</v>
       </c>
@@ -6010,7 +6009,7 @@
       <c r="P115" s="5"/>
       <c r="T115" s="4"/>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>4</v>
       </c>
@@ -6058,7 +6057,7 @@
       <c r="S116" s="7"/>
       <c r="T116" s="8"/>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>4</v>
       </c>
@@ -6078,7 +6077,7 @@
       <c r="M117" s="89"/>
       <c r="N117" s="90"/>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>4</v>
       </c>
@@ -6094,7 +6093,7 @@
       <c r="F118" s="18">
         <v>106</v>
       </c>
-      <c r="G118" s="7">
+      <c r="G118" s="18">
         <v>107</v>
       </c>
       <c r="H118" s="7"/>
@@ -6103,13 +6102,13 @@
       <c r="M118" s="89"/>
       <c r="N118" s="90"/>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C119" s="89"/>
       <c r="D119" s="90"/>
       <c r="M119" s="89"/>
       <c r="N119" s="90"/>
     </row>
-    <row r="121" spans="1:20" ht="18" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B121" s="14" t="s">
         <v>0</v>
       </c>
@@ -6121,7 +6120,7 @@
       <c r="F121" s="1"/>
       <c r="G121" s="1"/>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
       <c r="D122" s="1"/>
@@ -6129,34 +6128,34 @@
       <c r="F122" s="1"/>
       <c r="G122" s="1"/>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B123" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C123" s="40"/>
       <c r="D123" s="9"/>
-      <c r="F123" s="101" t="s">
+      <c r="F123" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="G123" s="102"/>
-      <c r="H123" s="102"/>
-      <c r="I123" s="102"/>
-      <c r="J123" s="102"/>
+      <c r="G123" s="103"/>
+      <c r="H123" s="103"/>
+      <c r="I123" s="103"/>
+      <c r="J123" s="103"/>
       <c r="L123" s="9" t="s">
         <v>2</v>
       </c>
       <c r="M123" s="40"/>
       <c r="N123" s="9"/>
       <c r="O123" s="33"/>
-      <c r="P123" s="101" t="s">
+      <c r="P123" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="Q123" s="102"/>
-      <c r="R123" s="102"/>
-      <c r="S123" s="102"/>
-      <c r="T123" s="102"/>
-    </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="Q123" s="103"/>
+      <c r="R123" s="103"/>
+      <c r="S123" s="103"/>
+      <c r="T123" s="103"/>
+    </row>
+    <row r="124" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B124" s="9" t="s">
         <v>10</v>
       </c>
@@ -6212,7 +6211,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>8</v>
       </c>
@@ -6251,7 +6250,7 @@
       <c r="S125" s="30"/>
       <c r="T125" s="31"/>
     </row>
-    <row r="126" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>8</v>
       </c>
@@ -6288,7 +6287,7 @@
       </c>
       <c r="T126" s="4"/>
     </row>
-    <row r="127" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>8</v>
       </c>
@@ -6341,7 +6340,7 @@
       <c r="S127" s="30"/>
       <c r="T127" s="31"/>
     </row>
-    <row r="128" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>8</v>
       </c>
@@ -6393,7 +6392,7 @@
       </c>
       <c r="T128" s="4"/>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>8</v>
       </c>
@@ -6445,7 +6444,7 @@
       </c>
       <c r="T129" s="4"/>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>8</v>
       </c>
@@ -6499,7 +6498,7 @@
       <c r="S130" s="30"/>
       <c r="T130" s="31"/>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>8</v>
       </c>
@@ -6552,7 +6551,7 @@
       <c r="S131" s="30"/>
       <c r="T131" s="31"/>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>8</v>
       </c>
@@ -6606,7 +6605,7 @@
       <c r="S132" s="30"/>
       <c r="T132" s="31"/>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>8</v>
       </c>
@@ -6657,7 +6656,7 @@
       <c r="S133" s="30"/>
       <c r="T133" s="31"/>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>8</v>
       </c>
@@ -6709,7 +6708,7 @@
       </c>
       <c r="T134" s="4"/>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>8</v>
       </c>
@@ -6761,7 +6760,7 @@
       </c>
       <c r="T135" s="4"/>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>8</v>
       </c>
@@ -6813,7 +6812,7 @@
       </c>
       <c r="T136" s="4"/>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>8</v>
       </c>
@@ -6866,7 +6865,7 @@
       </c>
       <c r="T137" s="4"/>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>8</v>
       </c>
@@ -6920,7 +6919,7 @@
       </c>
       <c r="T138" s="4"/>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>8</v>
       </c>
@@ -6975,7 +6974,7 @@
       <c r="S139" s="30"/>
       <c r="T139" s="31"/>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>8</v>
       </c>
@@ -7013,7 +7012,7 @@
       <c r="P140" s="5"/>
       <c r="T140" s="4"/>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>8</v>
       </c>
@@ -7056,7 +7055,7 @@
       <c r="S141" s="7"/>
       <c r="T141" s="8"/>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B144" t="s">
         <v>40</v>
       </c>
@@ -7076,7 +7075,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="145" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B145" t="s">
         <v>41</v>
       </c>
@@ -7084,7 +7083,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="146" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B146">
         <v>125</v>
       </c>
@@ -7092,7 +7091,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="147" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B147">
         <v>126</v>
       </c>
@@ -7100,7 +7099,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="149" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B149" t="s">
         <v>42</v>
       </c>
@@ -7108,7 +7107,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="150" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B150" t="str">
         <f ca="1">"3,1,"&amp;INDIRECT(D144&amp;B146)&amp;","&amp;INDIRECT(D144&amp;B147)&amp;",0,-1,NONE,NONE,SO MINISCAN "&amp;A141&amp;"KHZ STARTING ORDER "&amp;INDIRECT(C144&amp;B146)&amp;" &amp; "&amp;INDIRECT(C144&amp;B147)</f>
         <v>3,1,220,221,0,-1,NONE,NONE,SO MINISCAN 8KHZ STARTING ORDER 110 &amp; 116</v>

</xml_diff>

<commit_message>
MTP109 done; MTP110 generated
</commit_message>
<xml_diff>
--- a/observations/calibrations/solar_calibrations.xlsx
+++ b/observations/calibrations/solar_calibrations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iant\Documents\PROGRAMS\nomad_obs\observations\calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F92D13-75E3-4898-8647-9031C2CBA073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75B9012A-CDD1-4052-B62A-B432C05A13F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1635" yWindow="1425" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -919,7 +919,7 @@
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1068,6 +1068,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="18" builtinId="30" customBuiltin="1"/>
@@ -1669,7 +1671,9 @@
       <c r="P11" s="15">
         <v>105</v>
       </c>
-      <c r="Q11" s="16"/>
+      <c r="Q11" s="15">
+        <v>109</v>
+      </c>
       <c r="R11" s="16"/>
       <c r="S11" s="16"/>
       <c r="T11" s="16"/>
@@ -5990,7 +5994,7 @@
       <c r="H115" s="3">
         <v>97</v>
       </c>
-      <c r="I115" s="3"/>
+      <c r="I115" s="104"/>
       <c r="J115" s="4"/>
       <c r="L115" s="5">
         <f t="shared" si="7"/>
@@ -6036,6 +6040,7 @@
       <c r="H116" s="3">
         <v>97</v>
       </c>
+      <c r="I116" s="105"/>
       <c r="J116" s="4"/>
       <c r="L116" s="6">
         <f>L115+3</f>
@@ -6073,6 +6078,12 @@
       <c r="F117" s="3">
         <v>106</v>
       </c>
+      <c r="G117" s="3">
+        <v>109</v>
+      </c>
+      <c r="H117" s="3">
+        <v>109</v>
+      </c>
       <c r="J117" s="4"/>
       <c r="M117" s="89"/>
       <c r="N117" s="90"/>
@@ -6096,8 +6107,12 @@
       <c r="G118" s="18">
         <v>107</v>
       </c>
-      <c r="H118" s="7"/>
-      <c r="I118" s="7"/>
+      <c r="H118" s="18">
+        <v>109</v>
+      </c>
+      <c r="I118" s="18">
+        <v>109</v>
+      </c>
       <c r="J118" s="8"/>
       <c r="M118" s="89"/>
       <c r="N118" s="90"/>

</xml_diff>

<commit_message>
MTP110 done. Py scripts renamed based on order
</commit_message>
<xml_diff>
--- a/observations/calibrations/solar_calibrations.xlsx
+++ b/observations/calibrations/solar_calibrations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iant\Documents\PROGRAMS\nomad_obs\observations\calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75B9012A-CDD1-4052-B62A-B432C05A13F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D3A557-EB85-49C5-92DB-E1938EED6B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -919,7 +919,7 @@
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1068,8 +1068,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="18" builtinId="30" customBuiltin="1"/>
@@ -1392,23 +1390,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AE150"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" customWidth="1"/>
-    <col min="5" max="5" width="21.7109375" customWidth="1"/>
-    <col min="12" max="12" width="16.85546875" customWidth="1"/>
-    <col min="13" max="13" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" customWidth="1"/>
+    <col min="12" max="12" width="16.88671875" customWidth="1"/>
+    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="21" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.28515625" customWidth="1"/>
-    <col min="23" max="23" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.33203125" customWidth="1"/>
+    <col min="23" max="23" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1416,12 +1414,12 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:31" ht="18" x14ac:dyDescent="0.35">
       <c r="W2" s="14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:31" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="14" t="s">
         <v>3</v>
       </c>
@@ -1434,7 +1432,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:31" x14ac:dyDescent="0.3">
       <c r="C4" s="13" t="s">
         <v>12</v>
       </c>
@@ -1473,7 +1471,7 @@
       <c r="AD4" s="71"/>
       <c r="AE4" s="65"/>
     </row>
-    <row r="5" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:31" x14ac:dyDescent="0.3">
       <c r="C5" s="19" t="s">
         <v>1</v>
       </c>
@@ -1513,9 +1511,12 @@
       <c r="O5" s="3">
         <v>92</v>
       </c>
+      <c r="P5" s="3">
+        <v>110</v>
+      </c>
       <c r="AE5" s="4"/>
     </row>
-    <row r="6" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:31" x14ac:dyDescent="0.3">
       <c r="C6" s="20" t="s">
         <v>2</v>
       </c>
@@ -1580,14 +1581,14 @@
       <c r="AD6" s="7"/>
       <c r="AE6" s="8"/>
     </row>
-    <row r="9" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:31" ht="18" x14ac:dyDescent="0.35">
       <c r="B9" s="14" t="s">
         <v>24</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:31" x14ac:dyDescent="0.3">
       <c r="C10" s="13" t="s">
         <v>12</v>
       </c>
@@ -1628,7 +1629,7 @@
       <c r="AD10" s="71"/>
       <c r="AE10" s="65"/>
     </row>
-    <row r="11" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:31" x14ac:dyDescent="0.3">
       <c r="C11" s="19" t="s">
         <v>34</v>
       </c>
@@ -1689,7 +1690,7 @@
       <c r="AD11" s="16"/>
       <c r="AE11" s="17"/>
     </row>
-    <row r="12" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:31" x14ac:dyDescent="0.3">
       <c r="C12" s="20" t="s">
         <v>36</v>
       </c>
@@ -1734,12 +1735,12 @@
       <c r="AD12" s="7"/>
       <c r="AE12" s="8"/>
     </row>
-    <row r="13" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:31" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:31" ht="18" x14ac:dyDescent="0.35">
       <c r="B15" s="14" t="s">
         <v>0</v>
       </c>
@@ -1753,12 +1754,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:31" x14ac:dyDescent="0.3">
       <c r="AC16" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B17" s="9" t="s">
         <v>1</v>
       </c>
@@ -1786,7 +1787,7 @@
       <c r="S17" s="103"/>
       <c r="T17" s="103"/>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B18" s="39" t="s">
         <v>10</v>
       </c>
@@ -1861,7 +1862,7 @@
       </c>
       <c r="AE18" s="9"/>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1</v>
       </c>
@@ -1916,7 +1917,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1</v>
       </c>
@@ -1965,7 +1966,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1</v>
       </c>
@@ -2012,7 +2013,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>1</v>
       </c>
@@ -2076,7 +2077,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>1</v>
       </c>
@@ -2125,7 +2126,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>1</v>
       </c>
@@ -2174,7 +2175,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>1</v>
       </c>
@@ -2234,7 +2235,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>1</v>
       </c>
@@ -2283,7 +2284,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>1</v>
       </c>
@@ -2335,7 +2336,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>1</v>
       </c>
@@ -2380,7 +2381,7 @@
       </c>
       <c r="Z28" s="55"/>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>1</v>
       </c>
@@ -2423,7 +2424,7 @@
       <c r="Y29" s="48"/>
       <c r="Z29" s="49"/>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>1</v>
       </c>
@@ -2472,7 +2473,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>1</v>
       </c>
@@ -2517,7 +2518,7 @@
       <c r="Y31" s="48"/>
       <c r="Z31" s="49"/>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>1</v>
       </c>
@@ -2569,7 +2570,7 @@
       <c r="Y32" s="48"/>
       <c r="Z32" s="49"/>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>1</v>
       </c>
@@ -2614,7 +2615,7 @@
       <c r="Y33" s="48"/>
       <c r="Z33" s="49"/>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>1</v>
       </c>
@@ -2666,7 +2667,7 @@
       <c r="Y34" s="48"/>
       <c r="Z34" s="49"/>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>1</v>
       </c>
@@ -2712,7 +2713,7 @@
       <c r="Y35" s="48"/>
       <c r="Z35" s="49"/>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>1</v>
       </c>
@@ -2757,7 +2758,7 @@
       <c r="Y36" s="48"/>
       <c r="Z36" s="49"/>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>1</v>
       </c>
@@ -2800,7 +2801,7 @@
       <c r="Y37" s="48"/>
       <c r="Z37" s="49"/>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>1</v>
       </c>
@@ -2843,7 +2844,7 @@
       <c r="Y38" s="48"/>
       <c r="Z38" s="49"/>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>1</v>
       </c>
@@ -2889,7 +2890,7 @@
       <c r="Y39" s="48"/>
       <c r="Z39" s="49"/>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>1</v>
       </c>
@@ -2932,7 +2933,7 @@
       <c r="Y40" s="48"/>
       <c r="Z40" s="49"/>
     </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>1</v>
       </c>
@@ -2982,7 +2983,7 @@
       <c r="Y41" s="48"/>
       <c r="Z41" s="49"/>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>1</v>
       </c>
@@ -3033,7 +3034,7 @@
       <c r="Y42" s="48"/>
       <c r="Z42" s="49"/>
     </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>1</v>
       </c>
@@ -3088,7 +3089,7 @@
       <c r="Y43" s="48"/>
       <c r="Z43" s="49"/>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>1</v>
       </c>
@@ -3135,7 +3136,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>1</v>
       </c>
@@ -3181,7 +3182,7 @@
       <c r="Y45" s="5"/>
       <c r="Z45" s="4"/>
     </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>1</v>
       </c>
@@ -3222,7 +3223,7 @@
       <c r="Y46" s="5"/>
       <c r="Z46" s="4"/>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>1</v>
       </c>
@@ -3266,7 +3267,7 @@
       <c r="Y47" s="5"/>
       <c r="Z47" s="4"/>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>1</v>
       </c>
@@ -3317,7 +3318,7 @@
       <c r="Y48" s="5"/>
       <c r="Z48" s="4"/>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.3">
       <c r="W49" s="5">
         <v>4526.9799999999996</v>
       </c>
@@ -3327,7 +3328,7 @@
       <c r="Y49" s="6"/>
       <c r="Z49" s="8"/>
     </row>
-    <row r="50" spans="1:26" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:26" ht="18" x14ac:dyDescent="0.35">
       <c r="B50" s="14" t="s">
         <v>0</v>
       </c>
@@ -3339,7 +3340,7 @@
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
     </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
       <c r="D51" s="1"/>
@@ -3350,7 +3351,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B52" s="9" t="s">
         <v>1</v>
       </c>
@@ -3378,7 +3379,7 @@
       <c r="S52" s="103"/>
       <c r="T52" s="103"/>
     </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B53" s="9" t="s">
         <v>10</v>
       </c>
@@ -3434,7 +3435,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>2</v>
       </c>
@@ -3471,7 +3472,7 @@
       </c>
       <c r="T54" s="4"/>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>2</v>
       </c>
@@ -3508,7 +3509,7 @@
       <c r="P55" s="5"/>
       <c r="T55" s="4"/>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>2</v>
       </c>
@@ -3560,7 +3561,7 @@
       <c r="S56" s="30"/>
       <c r="T56" s="31"/>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>2</v>
       </c>
@@ -3597,7 +3598,7 @@
       <c r="P57" s="5"/>
       <c r="T57" s="4"/>
     </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>2</v>
       </c>
@@ -3634,7 +3635,7 @@
       <c r="P58" s="5"/>
       <c r="T58" s="4"/>
     </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>2</v>
       </c>
@@ -3675,7 +3676,7 @@
       </c>
       <c r="T59" s="4"/>
     </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>2</v>
       </c>
@@ -3712,7 +3713,7 @@
       <c r="P60" s="5"/>
       <c r="T60" s="4"/>
     </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>2</v>
       </c>
@@ -3764,7 +3765,7 @@
       <c r="S61" s="30"/>
       <c r="T61" s="31"/>
     </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>2</v>
       </c>
@@ -3801,7 +3802,7 @@
       <c r="P62" s="5"/>
       <c r="T62" s="4"/>
     </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>2</v>
       </c>
@@ -3853,7 +3854,7 @@
       <c r="S63" s="30"/>
       <c r="T63" s="31"/>
     </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>2</v>
       </c>
@@ -3890,7 +3891,7 @@
       <c r="P64" s="5"/>
       <c r="T64" s="4"/>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>2</v>
       </c>
@@ -3927,7 +3928,7 @@
       <c r="P65" s="35"/>
       <c r="T65" s="4"/>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>2</v>
       </c>
@@ -3964,7 +3965,7 @@
       <c r="P66" s="5"/>
       <c r="T66" s="4"/>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>2</v>
       </c>
@@ -4001,7 +4002,7 @@
       <c r="P67" s="5"/>
       <c r="T67" s="4"/>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>2</v>
       </c>
@@ -4053,7 +4054,7 @@
       <c r="S68" s="30"/>
       <c r="T68" s="31"/>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>2</v>
       </c>
@@ -4100,7 +4101,7 @@
       </c>
       <c r="T69" s="4"/>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>2</v>
       </c>
@@ -4141,7 +4142,7 @@
       </c>
       <c r="T70" s="4"/>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>2</v>
       </c>
@@ -4178,7 +4179,7 @@
       <c r="P71" s="5"/>
       <c r="T71" s="4"/>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>2</v>
       </c>
@@ -4215,7 +4216,7 @@
       <c r="P72" s="5"/>
       <c r="T72" s="4"/>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>2</v>
       </c>
@@ -4252,7 +4253,7 @@
       <c r="P73" s="5"/>
       <c r="T73" s="4"/>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>2</v>
       </c>
@@ -4289,7 +4290,7 @@
       <c r="P74" s="5"/>
       <c r="T74" s="4"/>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>2</v>
       </c>
@@ -4326,7 +4327,7 @@
       <c r="P75" s="5"/>
       <c r="T75" s="4"/>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>2</v>
       </c>
@@ -4367,7 +4368,7 @@
       </c>
       <c r="T76" s="4"/>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>2</v>
       </c>
@@ -4411,7 +4412,7 @@
       </c>
       <c r="T77" s="4"/>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>2</v>
       </c>
@@ -4448,7 +4449,7 @@
       <c r="P78" s="5"/>
       <c r="T78" s="4"/>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>2</v>
       </c>
@@ -4496,7 +4497,7 @@
       <c r="S79" s="30"/>
       <c r="T79" s="31"/>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>2</v>
       </c>
@@ -4533,7 +4534,7 @@
       <c r="P80" s="5"/>
       <c r="T80" s="4"/>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>2</v>
       </c>
@@ -4570,7 +4571,7 @@
       <c r="P81" s="5"/>
       <c r="T81" s="4"/>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>2</v>
       </c>
@@ -4613,7 +4614,7 @@
       <c r="S82" s="7"/>
       <c r="T82" s="8"/>
     </row>
-    <row r="84" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:20" ht="18" x14ac:dyDescent="0.35">
       <c r="B84" s="14" t="s">
         <v>0</v>
       </c>
@@ -4627,7 +4628,7 @@
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
       <c r="D85" s="1"/>
@@ -4635,7 +4636,7 @@
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B86" s="9" t="s">
         <v>1</v>
       </c>
@@ -4663,7 +4664,7 @@
       <c r="S86" s="103"/>
       <c r="T86" s="103"/>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B87" s="9" t="s">
         <v>10</v>
       </c>
@@ -4719,7 +4720,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>4</v>
       </c>
@@ -4760,7 +4761,7 @@
       <c r="S88" s="16"/>
       <c r="T88" s="17"/>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>4</v>
       </c>
@@ -4804,7 +4805,7 @@
       </c>
       <c r="T89" s="4"/>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>4</v>
       </c>
@@ -4856,7 +4857,7 @@
       <c r="S90" s="30"/>
       <c r="T90" s="31"/>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>4</v>
       </c>
@@ -4904,7 +4905,7 @@
       </c>
       <c r="T91" s="4"/>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>4</v>
       </c>
@@ -4943,7 +4944,7 @@
       <c r="P92" s="5"/>
       <c r="T92" s="4"/>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>4</v>
       </c>
@@ -4982,7 +4983,7 @@
       <c r="P93" s="5"/>
       <c r="T93" s="4"/>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>4</v>
       </c>
@@ -5026,7 +5027,7 @@
       </c>
       <c r="T94" s="4"/>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>4</v>
       </c>
@@ -5080,7 +5081,7 @@
       <c r="S95" s="30"/>
       <c r="T95" s="31"/>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>4</v>
       </c>
@@ -5121,7 +5122,7 @@
       </c>
       <c r="T96" s="4"/>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>4</v>
       </c>
@@ -5173,7 +5174,7 @@
       <c r="S97" s="30"/>
       <c r="T97" s="31"/>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>4</v>
       </c>
@@ -5222,7 +5223,7 @@
       <c r="S98" s="30"/>
       <c r="T98" s="31"/>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>4</v>
       </c>
@@ -5263,7 +5264,7 @@
       </c>
       <c r="T99" s="4"/>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>4</v>
       </c>
@@ -5304,7 +5305,7 @@
       </c>
       <c r="T100" s="4"/>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>4</v>
       </c>
@@ -5345,7 +5346,7 @@
       </c>
       <c r="T101" s="4"/>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>4</v>
       </c>
@@ -5397,7 +5398,7 @@
       <c r="S102" s="30"/>
       <c r="T102" s="31"/>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>4</v>
       </c>
@@ -5446,7 +5447,7 @@
       </c>
       <c r="T103" s="4"/>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>4</v>
       </c>
@@ -5492,7 +5493,7 @@
       </c>
       <c r="T104" s="4"/>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>4</v>
       </c>
@@ -5536,7 +5537,7 @@
       </c>
       <c r="T105" s="4"/>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>4</v>
       </c>
@@ -5580,7 +5581,7 @@
       </c>
       <c r="T106" s="4"/>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>4</v>
       </c>
@@ -5624,7 +5625,7 @@
       </c>
       <c r="T107" s="4"/>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>4</v>
       </c>
@@ -5668,7 +5669,7 @@
       </c>
       <c r="T108" s="4"/>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>4</v>
       </c>
@@ -5712,7 +5713,7 @@
       </c>
       <c r="T109" s="4"/>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>4</v>
       </c>
@@ -5756,7 +5757,7 @@
       </c>
       <c r="T110" s="4"/>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>4</v>
       </c>
@@ -5809,7 +5810,7 @@
       </c>
       <c r="T111" s="4"/>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>4</v>
       </c>
@@ -5862,7 +5863,7 @@
       </c>
       <c r="T112" s="4"/>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>4</v>
       </c>
@@ -5916,7 +5917,7 @@
       <c r="S113" s="30"/>
       <c r="T113" s="31"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>4</v>
       </c>
@@ -5967,7 +5968,7 @@
       <c r="Q114" s="73"/>
       <c r="T114" s="4"/>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>4</v>
       </c>
@@ -5994,7 +5995,6 @@
       <c r="H115" s="3">
         <v>97</v>
       </c>
-      <c r="I115" s="104"/>
       <c r="J115" s="4"/>
       <c r="L115" s="5">
         <f t="shared" si="7"/>
@@ -6013,7 +6013,7 @@
       <c r="P115" s="5"/>
       <c r="T115" s="4"/>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>4</v>
       </c>
@@ -6040,7 +6040,6 @@
       <c r="H116" s="3">
         <v>97</v>
       </c>
-      <c r="I116" s="105"/>
       <c r="J116" s="4"/>
       <c r="L116" s="6">
         <f>L115+3</f>
@@ -6062,7 +6061,7 @@
       <c r="S116" s="7"/>
       <c r="T116" s="8"/>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>4</v>
       </c>
@@ -6088,7 +6087,7 @@
       <c r="M117" s="89"/>
       <c r="N117" s="90"/>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>4</v>
       </c>
@@ -6117,13 +6116,13 @@
       <c r="M118" s="89"/>
       <c r="N118" s="90"/>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
       <c r="C119" s="89"/>
       <c r="D119" s="90"/>
       <c r="M119" s="89"/>
       <c r="N119" s="90"/>
     </row>
-    <row r="121" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:20" ht="18" x14ac:dyDescent="0.35">
       <c r="B121" s="14" t="s">
         <v>0</v>
       </c>
@@ -6135,7 +6134,7 @@
       <c r="F121" s="1"/>
       <c r="G121" s="1"/>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
       <c r="D122" s="1"/>
@@ -6143,7 +6142,7 @@
       <c r="F122" s="1"/>
       <c r="G122" s="1"/>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B123" s="9" t="s">
         <v>1</v>
       </c>
@@ -6170,7 +6169,7 @@
       <c r="S123" s="103"/>
       <c r="T123" s="103"/>
     </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B124" s="9" t="s">
         <v>10</v>
       </c>
@@ -6226,7 +6225,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>8</v>
       </c>
@@ -6265,7 +6264,7 @@
       <c r="S125" s="30"/>
       <c r="T125" s="31"/>
     </row>
-    <row r="126" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>8</v>
       </c>
@@ -6302,7 +6301,7 @@
       </c>
       <c r="T126" s="4"/>
     </row>
-    <row r="127" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>8</v>
       </c>
@@ -6355,7 +6354,7 @@
       <c r="S127" s="30"/>
       <c r="T127" s="31"/>
     </row>
-    <row r="128" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>8</v>
       </c>
@@ -6407,7 +6406,7 @@
       </c>
       <c r="T128" s="4"/>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>8</v>
       </c>
@@ -6459,7 +6458,7 @@
       </c>
       <c r="T129" s="4"/>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>8</v>
       </c>
@@ -6513,7 +6512,7 @@
       <c r="S130" s="30"/>
       <c r="T130" s="31"/>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>8</v>
       </c>
@@ -6566,7 +6565,7 @@
       <c r="S131" s="30"/>
       <c r="T131" s="31"/>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>8</v>
       </c>
@@ -6620,7 +6619,7 @@
       <c r="S132" s="30"/>
       <c r="T132" s="31"/>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>8</v>
       </c>
@@ -6671,7 +6670,7 @@
       <c r="S133" s="30"/>
       <c r="T133" s="31"/>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>8</v>
       </c>
@@ -6723,7 +6722,7 @@
       </c>
       <c r="T134" s="4"/>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>8</v>
       </c>
@@ -6775,7 +6774,7 @@
       </c>
       <c r="T135" s="4"/>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>8</v>
       </c>
@@ -6827,7 +6826,7 @@
       </c>
       <c r="T136" s="4"/>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>8</v>
       </c>
@@ -6880,7 +6879,7 @@
       </c>
       <c r="T137" s="4"/>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>8</v>
       </c>
@@ -6934,7 +6933,7 @@
       </c>
       <c r="T138" s="4"/>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>8</v>
       </c>
@@ -6989,7 +6988,7 @@
       <c r="S139" s="30"/>
       <c r="T139" s="31"/>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>8</v>
       </c>
@@ -7027,7 +7026,7 @@
       <c r="P140" s="5"/>
       <c r="T140" s="4"/>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>8</v>
       </c>
@@ -7070,7 +7069,7 @@
       <c r="S141" s="7"/>
       <c r="T141" s="8"/>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>40</v>
       </c>
@@ -7090,7 +7089,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="145" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>41</v>
       </c>
@@ -7098,7 +7097,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="146" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B146">
         <v>125</v>
       </c>
@@ -7106,7 +7105,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="147" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B147">
         <v>126</v>
       </c>
@@ -7114,7 +7113,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="149" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>42</v>
       </c>
@@ -7122,7 +7121,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="150" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B150" t="str">
         <f ca="1">"3,1,"&amp;INDIRECT(D144&amp;B146)&amp;","&amp;INDIRECT(D144&amp;B147)&amp;",0,-1,NONE,NONE,SO MINISCAN "&amp;A141&amp;"KHZ STARTING ORDER "&amp;INDIRECT(C144&amp;B146)&amp;" &amp; "&amp;INDIRECT(C144&amp;B147)</f>
         <v>3,1,220,221,0,-1,NONE,NONE,SO MINISCAN 8KHZ STARTING ORDER 110 &amp; 116</v>

</xml_diff>

<commit_message>
MTP111 done; MTP112 overview files downloaded
</commit_message>
<xml_diff>
--- a/observations/calibrations/solar_calibrations.xlsx
+++ b/observations/calibrations/solar_calibrations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iant\Documents\PROGRAMS\nomad_obs\observations\calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D3A557-EB85-49C5-92DB-E1938EED6B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C00FA75-1BC2-4A80-8A2C-7EAACA457B77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -919,7 +919,7 @@
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1068,6 +1068,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="18" builtinId="30" customBuiltin="1"/>
@@ -1390,23 +1392,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AE150"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" customWidth="1"/>
-    <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.109375" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" customWidth="1"/>
+    <col min="13" max="13" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="21" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.33203125" customWidth="1"/>
-    <col min="23" max="23" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.28515625" customWidth="1"/>
+    <col min="23" max="23" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:31" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1414,12 +1416,12 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="2:31" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
       <c r="W2" s="14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="2:31" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B3" s="14" t="s">
         <v>3</v>
       </c>
@@ -1432,7 +1434,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C4" s="13" t="s">
         <v>12</v>
       </c>
@@ -1471,7 +1473,7 @@
       <c r="AD4" s="71"/>
       <c r="AE4" s="65"/>
     </row>
-    <row r="5" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C5" s="19" t="s">
         <v>1</v>
       </c>
@@ -1516,7 +1518,7 @@
       </c>
       <c r="AE5" s="4"/>
     </row>
-    <row r="6" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C6" s="20" t="s">
         <v>2</v>
       </c>
@@ -1581,14 +1583,14 @@
       <c r="AD6" s="7"/>
       <c r="AE6" s="8"/>
     </row>
-    <row r="9" spans="2:31" ht="18" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="14" t="s">
         <v>24</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C10" s="13" t="s">
         <v>12</v>
       </c>
@@ -1629,7 +1631,7 @@
       <c r="AD10" s="71"/>
       <c r="AE10" s="65"/>
     </row>
-    <row r="11" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C11" s="19" t="s">
         <v>34</v>
       </c>
@@ -1690,7 +1692,7 @@
       <c r="AD11" s="16"/>
       <c r="AE11" s="17"/>
     </row>
-    <row r="12" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C12" s="20" t="s">
         <v>36</v>
       </c>
@@ -1735,12 +1737,12 @@
       <c r="AD12" s="7"/>
       <c r="AE12" s="8"/>
     </row>
-    <row r="13" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:31" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="2:31" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:31" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B15" s="14" t="s">
         <v>0</v>
       </c>
@@ -1754,12 +1756,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="2:31" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:31" x14ac:dyDescent="0.25">
       <c r="AC16" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
         <v>1</v>
       </c>
@@ -1787,7 +1789,7 @@
       <c r="S17" s="103"/>
       <c r="T17" s="103"/>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B18" s="39" t="s">
         <v>10</v>
       </c>
@@ -1862,7 +1864,7 @@
       </c>
       <c r="AE18" s="9"/>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1</v>
       </c>
@@ -1917,7 +1919,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1</v>
       </c>
@@ -1966,7 +1968,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1</v>
       </c>
@@ -2013,7 +2015,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1</v>
       </c>
@@ -2077,7 +2079,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1</v>
       </c>
@@ -2126,7 +2128,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1</v>
       </c>
@@ -2175,7 +2177,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1</v>
       </c>
@@ -2235,7 +2237,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1</v>
       </c>
@@ -2284,7 +2286,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1</v>
       </c>
@@ -2336,7 +2338,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1</v>
       </c>
@@ -2381,7 +2383,7 @@
       </c>
       <c r="Z28" s="55"/>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1</v>
       </c>
@@ -2424,7 +2426,7 @@
       <c r="Y29" s="48"/>
       <c r="Z29" s="49"/>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1</v>
       </c>
@@ -2473,7 +2475,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>1</v>
       </c>
@@ -2518,7 +2520,7 @@
       <c r="Y31" s="48"/>
       <c r="Z31" s="49"/>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>1</v>
       </c>
@@ -2570,7 +2572,7 @@
       <c r="Y32" s="48"/>
       <c r="Z32" s="49"/>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>1</v>
       </c>
@@ -2615,7 +2617,7 @@
       <c r="Y33" s="48"/>
       <c r="Z33" s="49"/>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>1</v>
       </c>
@@ -2667,7 +2669,7 @@
       <c r="Y34" s="48"/>
       <c r="Z34" s="49"/>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>1</v>
       </c>
@@ -2713,7 +2715,7 @@
       <c r="Y35" s="48"/>
       <c r="Z35" s="49"/>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>1</v>
       </c>
@@ -2758,7 +2760,7 @@
       <c r="Y36" s="48"/>
       <c r="Z36" s="49"/>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>1</v>
       </c>
@@ -2801,7 +2803,7 @@
       <c r="Y37" s="48"/>
       <c r="Z37" s="49"/>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>1</v>
       </c>
@@ -2844,7 +2846,7 @@
       <c r="Y38" s="48"/>
       <c r="Z38" s="49"/>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>1</v>
       </c>
@@ -2890,7 +2892,7 @@
       <c r="Y39" s="48"/>
       <c r="Z39" s="49"/>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>1</v>
       </c>
@@ -2933,7 +2935,7 @@
       <c r="Y40" s="48"/>
       <c r="Z40" s="49"/>
     </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>1</v>
       </c>
@@ -2983,7 +2985,7 @@
       <c r="Y41" s="48"/>
       <c r="Z41" s="49"/>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>1</v>
       </c>
@@ -3034,7 +3036,7 @@
       <c r="Y42" s="48"/>
       <c r="Z42" s="49"/>
     </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>1</v>
       </c>
@@ -3089,7 +3091,7 @@
       <c r="Y43" s="48"/>
       <c r="Z43" s="49"/>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>1</v>
       </c>
@@ -3136,7 +3138,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>1</v>
       </c>
@@ -3182,7 +3184,7 @@
       <c r="Y45" s="5"/>
       <c r="Z45" s="4"/>
     </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>1</v>
       </c>
@@ -3223,7 +3225,7 @@
       <c r="Y46" s="5"/>
       <c r="Z46" s="4"/>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>1</v>
       </c>
@@ -3267,7 +3269,7 @@
       <c r="Y47" s="5"/>
       <c r="Z47" s="4"/>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>1</v>
       </c>
@@ -3318,7 +3320,7 @@
       <c r="Y48" s="5"/>
       <c r="Z48" s="4"/>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
       <c r="W49" s="5">
         <v>4526.9799999999996</v>
       </c>
@@ -3328,7 +3330,7 @@
       <c r="Y49" s="6"/>
       <c r="Z49" s="8"/>
     </row>
-    <row r="50" spans="1:26" ht="18" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:26" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B50" s="14" t="s">
         <v>0</v>
       </c>
@@ -3340,7 +3342,7 @@
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
     </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
       <c r="D51" s="1"/>
@@ -3351,7 +3353,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B52" s="9" t="s">
         <v>1</v>
       </c>
@@ -3379,7 +3381,7 @@
       <c r="S52" s="103"/>
       <c r="T52" s="103"/>
     </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B53" s="9" t="s">
         <v>10</v>
       </c>
@@ -3435,7 +3437,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2</v>
       </c>
@@ -3472,7 +3474,7 @@
       </c>
       <c r="T54" s="4"/>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2</v>
       </c>
@@ -3509,7 +3511,7 @@
       <c r="P55" s="5"/>
       <c r="T55" s="4"/>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2</v>
       </c>
@@ -3561,7 +3563,7 @@
       <c r="S56" s="30"/>
       <c r="T56" s="31"/>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>2</v>
       </c>
@@ -3598,7 +3600,7 @@
       <c r="P57" s="5"/>
       <c r="T57" s="4"/>
     </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>2</v>
       </c>
@@ -3635,7 +3637,7 @@
       <c r="P58" s="5"/>
       <c r="T58" s="4"/>
     </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>2</v>
       </c>
@@ -3676,7 +3678,7 @@
       </c>
       <c r="T59" s="4"/>
     </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>2</v>
       </c>
@@ -3713,7 +3715,7 @@
       <c r="P60" s="5"/>
       <c r="T60" s="4"/>
     </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>2</v>
       </c>
@@ -3765,7 +3767,7 @@
       <c r="S61" s="30"/>
       <c r="T61" s="31"/>
     </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>2</v>
       </c>
@@ -3802,7 +3804,7 @@
       <c r="P62" s="5"/>
       <c r="T62" s="4"/>
     </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>2</v>
       </c>
@@ -3854,7 +3856,7 @@
       <c r="S63" s="30"/>
       <c r="T63" s="31"/>
     </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>2</v>
       </c>
@@ -3891,7 +3893,7 @@
       <c r="P64" s="5"/>
       <c r="T64" s="4"/>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>2</v>
       </c>
@@ -3928,7 +3930,7 @@
       <c r="P65" s="35"/>
       <c r="T65" s="4"/>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>2</v>
       </c>
@@ -3965,7 +3967,7 @@
       <c r="P66" s="5"/>
       <c r="T66" s="4"/>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>2</v>
       </c>
@@ -4002,7 +4004,7 @@
       <c r="P67" s="5"/>
       <c r="T67" s="4"/>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>2</v>
       </c>
@@ -4054,7 +4056,7 @@
       <c r="S68" s="30"/>
       <c r="T68" s="31"/>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>2</v>
       </c>
@@ -4101,7 +4103,7 @@
       </c>
       <c r="T69" s="4"/>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>2</v>
       </c>
@@ -4142,7 +4144,7 @@
       </c>
       <c r="T70" s="4"/>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>2</v>
       </c>
@@ -4179,7 +4181,7 @@
       <c r="P71" s="5"/>
       <c r="T71" s="4"/>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>2</v>
       </c>
@@ -4216,7 +4218,7 @@
       <c r="P72" s="5"/>
       <c r="T72" s="4"/>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>2</v>
       </c>
@@ -4253,7 +4255,7 @@
       <c r="P73" s="5"/>
       <c r="T73" s="4"/>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>2</v>
       </c>
@@ -4290,7 +4292,7 @@
       <c r="P74" s="5"/>
       <c r="T74" s="4"/>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>2</v>
       </c>
@@ -4327,7 +4329,7 @@
       <c r="P75" s="5"/>
       <c r="T75" s="4"/>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>2</v>
       </c>
@@ -4368,7 +4370,7 @@
       </c>
       <c r="T76" s="4"/>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>2</v>
       </c>
@@ -4412,7 +4414,7 @@
       </c>
       <c r="T77" s="4"/>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>2</v>
       </c>
@@ -4449,7 +4451,7 @@
       <c r="P78" s="5"/>
       <c r="T78" s="4"/>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>2</v>
       </c>
@@ -4497,7 +4499,7 @@
       <c r="S79" s="30"/>
       <c r="T79" s="31"/>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>2</v>
       </c>
@@ -4534,7 +4536,7 @@
       <c r="P80" s="5"/>
       <c r="T80" s="4"/>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>2</v>
       </c>
@@ -4571,7 +4573,7 @@
       <c r="P81" s="5"/>
       <c r="T81" s="4"/>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>2</v>
       </c>
@@ -4614,7 +4616,7 @@
       <c r="S82" s="7"/>
       <c r="T82" s="8"/>
     </row>
-    <row r="84" spans="1:20" ht="18" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B84" s="14" t="s">
         <v>0</v>
       </c>
@@ -4628,7 +4630,7 @@
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
       <c r="D85" s="1"/>
@@ -4636,7 +4638,7 @@
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B86" s="9" t="s">
         <v>1</v>
       </c>
@@ -4664,7 +4666,7 @@
       <c r="S86" s="103"/>
       <c r="T86" s="103"/>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B87" s="9" t="s">
         <v>10</v>
       </c>
@@ -4720,7 +4722,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>4</v>
       </c>
@@ -4761,7 +4763,7 @@
       <c r="S88" s="16"/>
       <c r="T88" s="17"/>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>4</v>
       </c>
@@ -4805,7 +4807,7 @@
       </c>
       <c r="T89" s="4"/>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>4</v>
       </c>
@@ -4857,7 +4859,7 @@
       <c r="S90" s="30"/>
       <c r="T90" s="31"/>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>4</v>
       </c>
@@ -4905,7 +4907,7 @@
       </c>
       <c r="T91" s="4"/>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>4</v>
       </c>
@@ -4944,7 +4946,7 @@
       <c r="P92" s="5"/>
       <c r="T92" s="4"/>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>4</v>
       </c>
@@ -4983,7 +4985,7 @@
       <c r="P93" s="5"/>
       <c r="T93" s="4"/>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>4</v>
       </c>
@@ -5027,7 +5029,7 @@
       </c>
       <c r="T94" s="4"/>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>4</v>
       </c>
@@ -5081,7 +5083,7 @@
       <c r="S95" s="30"/>
       <c r="T95" s="31"/>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>4</v>
       </c>
@@ -5122,7 +5124,7 @@
       </c>
       <c r="T96" s="4"/>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>4</v>
       </c>
@@ -5174,7 +5176,7 @@
       <c r="S97" s="30"/>
       <c r="T97" s="31"/>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>4</v>
       </c>
@@ -5223,7 +5225,7 @@
       <c r="S98" s="30"/>
       <c r="T98" s="31"/>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>4</v>
       </c>
@@ -5264,7 +5266,7 @@
       </c>
       <c r="T99" s="4"/>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>4</v>
       </c>
@@ -5305,7 +5307,7 @@
       </c>
       <c r="T100" s="4"/>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>4</v>
       </c>
@@ -5346,7 +5348,7 @@
       </c>
       <c r="T101" s="4"/>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>4</v>
       </c>
@@ -5398,7 +5400,7 @@
       <c r="S102" s="30"/>
       <c r="T102" s="31"/>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>4</v>
       </c>
@@ -5447,7 +5449,7 @@
       </c>
       <c r="T103" s="4"/>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>4</v>
       </c>
@@ -5493,7 +5495,7 @@
       </c>
       <c r="T104" s="4"/>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>4</v>
       </c>
@@ -5537,7 +5539,7 @@
       </c>
       <c r="T105" s="4"/>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>4</v>
       </c>
@@ -5581,7 +5583,7 @@
       </c>
       <c r="T106" s="4"/>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>4</v>
       </c>
@@ -5625,7 +5627,7 @@
       </c>
       <c r="T107" s="4"/>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>4</v>
       </c>
@@ -5669,7 +5671,7 @@
       </c>
       <c r="T108" s="4"/>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>4</v>
       </c>
@@ -5713,7 +5715,7 @@
       </c>
       <c r="T109" s="4"/>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>4</v>
       </c>
@@ -5757,7 +5759,7 @@
       </c>
       <c r="T110" s="4"/>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>4</v>
       </c>
@@ -5810,7 +5812,7 @@
       </c>
       <c r="T111" s="4"/>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>4</v>
       </c>
@@ -5863,7 +5865,7 @@
       </c>
       <c r="T112" s="4"/>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>4</v>
       </c>
@@ -5917,7 +5919,7 @@
       <c r="S113" s="30"/>
       <c r="T113" s="31"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>4</v>
       </c>
@@ -5968,7 +5970,7 @@
       <c r="Q114" s="73"/>
       <c r="T114" s="4"/>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>4</v>
       </c>
@@ -6013,7 +6015,7 @@
       <c r="P115" s="5"/>
       <c r="T115" s="4"/>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>4</v>
       </c>
@@ -6061,7 +6063,7 @@
       <c r="S116" s="7"/>
       <c r="T116" s="8"/>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>4</v>
       </c>
@@ -6083,11 +6085,14 @@
       <c r="H117" s="3">
         <v>109</v>
       </c>
+      <c r="I117" s="104">
+        <v>111</v>
+      </c>
       <c r="J117" s="4"/>
       <c r="M117" s="89"/>
       <c r="N117" s="90"/>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>4</v>
       </c>
@@ -6112,17 +6117,19 @@
       <c r="I118" s="18">
         <v>109</v>
       </c>
-      <c r="J118" s="8"/>
+      <c r="J118" s="105">
+        <v>111</v>
+      </c>
       <c r="M118" s="89"/>
       <c r="N118" s="90"/>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C119" s="89"/>
       <c r="D119" s="90"/>
       <c r="M119" s="89"/>
       <c r="N119" s="90"/>
     </row>
-    <row r="121" spans="1:20" ht="18" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B121" s="14" t="s">
         <v>0</v>
       </c>
@@ -6134,7 +6141,7 @@
       <c r="F121" s="1"/>
       <c r="G121" s="1"/>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
       <c r="D122" s="1"/>
@@ -6142,7 +6149,7 @@
       <c r="F122" s="1"/>
       <c r="G122" s="1"/>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B123" s="9" t="s">
         <v>1</v>
       </c>
@@ -6169,7 +6176,7 @@
       <c r="S123" s="103"/>
       <c r="T123" s="103"/>
     </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B124" s="9" t="s">
         <v>10</v>
       </c>
@@ -6225,7 +6232,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>8</v>
       </c>
@@ -6264,7 +6271,7 @@
       <c r="S125" s="30"/>
       <c r="T125" s="31"/>
     </row>
-    <row r="126" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>8</v>
       </c>
@@ -6301,7 +6308,7 @@
       </c>
       <c r="T126" s="4"/>
     </row>
-    <row r="127" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>8</v>
       </c>
@@ -6354,7 +6361,7 @@
       <c r="S127" s="30"/>
       <c r="T127" s="31"/>
     </row>
-    <row r="128" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>8</v>
       </c>
@@ -6406,7 +6413,7 @@
       </c>
       <c r="T128" s="4"/>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>8</v>
       </c>
@@ -6458,7 +6465,7 @@
       </c>
       <c r="T129" s="4"/>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>8</v>
       </c>
@@ -6512,7 +6519,7 @@
       <c r="S130" s="30"/>
       <c r="T130" s="31"/>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>8</v>
       </c>
@@ -6565,7 +6572,7 @@
       <c r="S131" s="30"/>
       <c r="T131" s="31"/>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>8</v>
       </c>
@@ -6619,7 +6626,7 @@
       <c r="S132" s="30"/>
       <c r="T132" s="31"/>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>8</v>
       </c>
@@ -6670,7 +6677,7 @@
       <c r="S133" s="30"/>
       <c r="T133" s="31"/>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>8</v>
       </c>
@@ -6722,7 +6729,7 @@
       </c>
       <c r="T134" s="4"/>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>8</v>
       </c>
@@ -6774,7 +6781,7 @@
       </c>
       <c r="T135" s="4"/>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>8</v>
       </c>
@@ -6826,7 +6833,7 @@
       </c>
       <c r="T136" s="4"/>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>8</v>
       </c>
@@ -6879,7 +6886,7 @@
       </c>
       <c r="T137" s="4"/>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>8</v>
       </c>
@@ -6933,7 +6940,7 @@
       </c>
       <c r="T138" s="4"/>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>8</v>
       </c>
@@ -6988,7 +6995,7 @@
       <c r="S139" s="30"/>
       <c r="T139" s="31"/>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>8</v>
       </c>
@@ -7009,6 +7016,9 @@
       </c>
       <c r="G140" s="3">
         <v>101</v>
+      </c>
+      <c r="H140" s="3">
+        <v>111</v>
       </c>
       <c r="J140" s="4"/>
       <c r="L140" s="5">
@@ -7026,7 +7036,7 @@
       <c r="P140" s="5"/>
       <c r="T140" s="4"/>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>8</v>
       </c>
@@ -7048,7 +7058,9 @@
       <c r="G141" s="18">
         <v>101</v>
       </c>
-      <c r="H141" s="7"/>
+      <c r="H141" s="18">
+        <v>111</v>
+      </c>
       <c r="I141" s="7"/>
       <c r="J141" s="8"/>
       <c r="L141" s="6">
@@ -7069,7 +7081,7 @@
       <c r="S141" s="7"/>
       <c r="T141" s="8"/>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B144" t="s">
         <v>40</v>
       </c>
@@ -7089,7 +7101,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="145" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B145" t="s">
         <v>41</v>
       </c>
@@ -7097,7 +7109,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="146" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B146">
         <v>125</v>
       </c>
@@ -7105,7 +7117,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="147" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B147">
         <v>126</v>
       </c>
@@ -7113,7 +7125,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="149" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B149" t="s">
         <v>42</v>
       </c>
@@ -7121,7 +7133,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="150" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B150" t="str">
         <f ca="1">"3,1,"&amp;INDIRECT(D144&amp;B146)&amp;","&amp;INDIRECT(D144&amp;B147)&amp;",0,-1,NONE,NONE,SO MINISCAN "&amp;A141&amp;"KHZ STARTING ORDER "&amp;INDIRECT(C144&amp;B146)&amp;" &amp; "&amp;INDIRECT(C144&amp;B147)</f>
         <v>3,1,220,221,0,-1,NONE,NONE,SO MINISCAN 8KHZ STARTING ORDER 110 &amp; 116</v>

</xml_diff>